<commit_message>
fix: repara el XML de la plantilla y quita el giro de drones
</commit_message>
<xml_diff>
--- a/docs/Plantilla_Captura_Reporteria_v1.xlsx
+++ b/docs/Plantilla_Captura_Reporteria_v1.xlsx
@@ -1345,12 +1345,14 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>13</v>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Use las listas desplegables donde existan: evitan errores de dedo (ej. 'Accesorios' vs 'Accesorio' en linea). El modelo es texto libre: el sistema ignora mayusculas y espacios sobrantes al agrupar, pero no une nombres escritos distinto; escribalo siempre igual.</t>
+        </is>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1511,7 +1513,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1519,21 +1521,18 @@
         <v>45</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E1" s="0" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F1" s="0" t="s">
-        <v>50</v>
-      </c>
-      <c r="G1" s="0" t="s">
         <v>51</v>
       </c>
     </row>
@@ -1542,21 +1541,18 @@
         <v>52</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>53</v>
+        <v>32</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>32</v>
+        <v>54</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>56</v>
-      </c>
-      <c r="G2" s="0" t="s">
         <v>57</v>
       </c>
     </row>
@@ -1565,18 +1561,15 @@
         <v>58</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>61</v>
-      </c>
-      <c r="E3" s="0" t="s">
         <v>62</v>
       </c>
-      <c r="G3" s="0" t="s">
+      <c r="F3" s="0" t="s">
         <v>63</v>
       </c>
     </row>
@@ -1584,13 +1577,10 @@
       <c r="A4" s="0" t="s">
         <v>64</v>
       </c>
-      <c r="B4" s="0" t="s">
-        <v>65</v>
-      </c>
-      <c r="E4" s="0" t="s">
+      <c r="D4" s="0" t="s">
         <v>66</v>
       </c>
-      <c r="G4" s="0" t="s">
+      <c r="F4" s="0" t="s">
         <v>67</v>
       </c>
     </row>
@@ -1598,13 +1588,10 @@
       <c r="A5" s="0" t="s">
         <v>68</v>
       </c>
-      <c r="B5" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="E5" s="0" t="s">
+      <c r="D5" s="0" t="s">
         <v>70</v>
       </c>
-      <c r="G5" s="0" t="s">
+      <c r="F5" s="0" t="s">
         <v>71</v>
       </c>
     </row>
@@ -1612,44 +1599,32 @@
       <c r="A6" s="0" t="s">
         <v>72</v>
       </c>
-      <c r="B6" s="0" t="s">
-        <v>73</v>
-      </c>
-      <c r="E6" s="0" t="s">
+      <c r="D6" s="0" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="0" t="s">
-        <v>75</v>
-      </c>
-      <c r="E7" s="0" t="s">
+      <c r="D7" s="0" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="0" t="s">
-        <v>77</v>
-      </c>
-      <c r="E8" s="0" t="s">
+      <c r="D8" s="0" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="0" t="s">
-        <v>79</v>
-      </c>
-      <c r="E9" s="0" t="s">
+      <c r="D9" s="0" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E10" s="0" t="s">
+      <c r="D10" s="0" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E11" s="0" t="s">
+      <c r="D11" s="0" t="s">
         <v>82</v>
       </c>
     </row>
@@ -1664,16 +1639,4240 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="UTF-8" standalone="yes"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006"><sheetPr filterMode="false"><pageSetUpPr fitToPage="false"/></sheetPr><dimension ref="A1:R301"/><sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"></sheetFormatPr><cols><col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/><col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/><col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13"/><col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="34"/><col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="17"/><col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18"/><col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="15"/><col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="12"/><col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="13"/><col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="11"/><col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="12"/><col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="16"/><col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="15"/><col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="11"/><col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="16" style="0" width="15"/><col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="40"/></cols><sheetData><row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"><c r="A1" s="6" t="s"><v>83</v></c><c r="B1" s="6" t="s"><v>84</v></c><c r="C1" s="6" t="s"><v>85</v></c><c r="D1" s="6" t="s"><v>86</v></c><c r="E1" s="6" t="s"><v>87</v></c><c r="F1" s="6" t="s"><v>88</v></c><c r="G1" s="6" t="s"><v>89</v></c><c r="H1" s="6" t="s"><v>90</v></c><c r="I1" s="6" t="s"><v>91</v></c><c r="J1" s="6" t="s"><v>92</v></c><c r="K1" s="6" t="s"><v>93</v></c><c r="L1" s="6" t="s"><v>94</v></c><c r="M1" s="6" t="s"><v>95</v></c><c r="N1" s="6" t="s"><v>96</v></c><c r="O1" s="6" t="s"><v>97</v></c><c r="P1" s="6" t="s"><v>98</v></c><c r="Q1" s="6" t="s"><v>99</v></c><c r="R1" s="6" t="s"><v>100</v></c></row><row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A2" s="7" t="s"><v>101</v></c><c r="B2" s="7" t="s"><v>102</v></c><c r="C2" s="7" t="s"><v>45</v></c><c r="D2" s="7" t="s"><v>103</v></c><c r="E2" s="7" t="s"><v>59</v></c><c r="F2" s="7" t="s"><v>104</v></c><c r="G2" s="8" t="n"><v>200000</v></c><c r="H2" s="8" t="n"><v>260000</v></c><c r="I2" s="9" t="n"><v>0.05</v></c><c r="J2" s="7" t="s"><v>48</v></c><c r="K2" s="7" t="n"><v>90</v></c><c r="L2" s="7" t="s"><v>32</v></c><c r="M2" s="7" t="s"><v>105</v></c><c r="N2" s="10" t="n"><f aca="false">IFERROR(H2-G2,&quot;&quot;)</f><v>60000</v></c><c r="O2" s="11" t="n"><f aca="false">IFERROR(N2/H2,&quot;&quot;)</f><v>0.230769230769231</v></c><c r="P2" s="10" t="n"><f aca="false">IFERROR(SUMIF(cobranza!$B$3:$B$1000,A2,cobranza!$D$3:$D$1000),0)</f><v>0</v></c><c r="Q2" s="10" t="n"><f aca="false">IFERROR(H2-P2,&quot;&quot;)</f><v>260000</v></c><c r="R2" s="12" t="s"><v>106</v></c></row><row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A3" s="18"/><row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A4" s="18"/><row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A5" s="18"/><row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A6" s="18"/><row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A7" s="18"/><row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A8" s="18"/><row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A9" s="18"/><row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A10" s="18"/><row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A11" s="18"/><row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A12" s="18"/><row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A13" s="18"/><row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A14" s="18"/><row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A15" s="18"/><row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A16" s="18"/><row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A17" s="18"/><row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A18" s="18"/><row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A19" s="18"/><row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A20" s="18"/><row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A21" s="18"/><row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A22" s="18"/><row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A23" s="18"/><row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A24" s="18"/><row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A25" s="18"/><row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A26" s="18"/><row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A27" s="18"/><row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A28" s="18"/><row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A29" s="18"/><row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A30" s="18"/><row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A31" s="18"/><row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A32" s="18"/><row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A33" s="18"/><row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A34" s="18"/><row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A35" s="18"/><row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A36" s="18"/><row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A37" s="18"/><row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A38" s="18"/><row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A39" s="18"/><row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A40" s="18"/><row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A41" s="18"/><row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A42" s="18"/><row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A43" s="18"/><row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A44" s="18"/><row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A45" s="18"/><row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A46" s="18"/><row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A47" s="18"/><row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A48" s="18"/><row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A49" s="18"/><row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A50" s="18"/><row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A51" s="18"/><row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A52" s="18"/><row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A53" s="18"/><row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A54" s="18"/><row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A55" s="18"/><row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A56" s="18"/><row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A57" s="18"/><row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A58" s="18"/><row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A59" s="18"/><row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A60" s="18"/><row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A61" s="18"/><row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A62" s="18"/><row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A63" s="18"/><row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A64" s="18"/><row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A65" s="18"/><row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A66" s="18"/><row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A67" s="18"/><row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A68" s="18"/><row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A69" s="18"/><row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A70" s="18"/><row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A71" s="18"/><row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A72" s="18"/><row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A73" s="18"/><row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A74" s="18"/><row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A75" s="18"/><row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A76" s="18"/><row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A77" s="18"/><row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A78" s="18"/><row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A79" s="18"/><row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A80" s="18"/><row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A81" s="18"/><row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A82" s="18"/><row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A83" s="18"/><row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A84" s="18"/><row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A85" s="18"/><row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A86" s="18"/><row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A87" s="18"/><row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A88" s="18"/><row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A89" s="18"/><row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A90" s="18"/><row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A91" s="18"/><row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A92" s="18"/><row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A93" s="18"/><row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A94" s="18"/><row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A95" s="18"/><row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A96" s="18"/><row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A97" s="18"/><row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A98" s="18"/><row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A99" s="18"/><row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A100" s="18"/><row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A101" s="18"/><row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A102" s="18"/><row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A103" s="18"/><row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A104" s="18"/><row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A105" s="18"/><row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A106" s="18"/><row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A107" s="18"/><row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A108" s="18"/><row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A109" s="18"/><row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A110" s="18"/><row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A111" s="18"/><row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A112" s="18"/><row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A113" s="18"/><row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A114" s="18"/><row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A115" s="18"/><row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A116" s="18"/><row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A117" s="18"/><row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A118" s="18"/><row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A119" s="18"/><row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A120" s="18"/><row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A121" s="18"/><row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A122" s="18"/><row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A123" s="18"/><row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A124" s="18"/><row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A125" s="18"/><row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A126" s="18"/><row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A127" s="18"/><row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A128" s="18"/><row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A129" s="18"/><row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A130" s="18"/><row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A131" s="18"/><row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A132" s="18"/><row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A133" s="18"/><row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A134" s="18"/><row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A135" s="18"/><row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A136" s="18"/><row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A137" s="18"/><row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A138" s="18"/><row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A139" s="18"/><row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A140" s="18"/><row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A141" s="18"/><row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A142" s="18"/><row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A143" s="18"/><row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A144" s="18"/><row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A145" s="18"/><row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A146" s="18"/><row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A147" s="18"/><row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A148" s="18"/><row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A149" s="18"/><row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A150" s="18"/><row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A151" s="18"/><row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A152" s="18"/><row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A153" s="18"/><row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A154" s="18"/><row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A155" s="18"/><row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A156" s="18"/><row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A157" s="18"/><row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A158" s="18"/><row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A159" s="18"/><row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A160" s="18"/><row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A161" s="18"/><row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A162" s="18"/><row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A163" s="18"/><row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A164" s="18"/><row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A165" s="18"/><row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A166" s="18"/><row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A167" s="18"/><row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A168" s="18"/><row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A169" s="18"/><row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A170" s="18"/><row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A171" s="18"/><row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A172" s="18"/><row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A173" s="18"/><row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A174" s="18"/><row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A175" s="18"/><row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A176" s="18"/><row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A177" s="18"/><row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A178" s="18"/><row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A179" s="18"/><row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A180" s="18"/><row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A181" s="18"/><row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A182" s="18"/><row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A183" s="18"/><row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A184" s="18"/><row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A185" s="18"/><row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A186" s="18"/><row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A187" s="18"/><row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A188" s="18"/><row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A189" s="18"/><row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A190" s="18"/><row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A191" s="18"/><row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A192" s="18"/><row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A193" s="18"/><row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A194" s="18"/><row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A195" s="18"/><row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A196" s="18"/><row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A197" s="18"/><row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A198" s="18"/><row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A199" s="18"/><row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A200" s="18"/><row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A201" s="18"/><row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A202" s="18"/><row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A203" s="18"/><row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A204" s="18"/><row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A205" s="18"/><row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A206" s="18"/><row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A207" s="18"/><row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A208" s="18"/><row r="209" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A209" s="18"/><row r="210" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A210" s="18"/><row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A211" s="18"/><row r="212" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A212" s="18"/><row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A213" s="18"/><row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A214" s="18"/><row r="215" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A215" s="18"/><row r="216" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A216" s="18"/><row r="217" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A217" s="18"/><row r="218" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A218" s="18"/><row r="219" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A219" s="18"/><row r="220" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A220" s="18"/><row r="221" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A221" s="18"/><row r="222" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A222" s="18"/><row r="223" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A223" s="18"/><row r="224" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A224" s="18"/><row r="225" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A225" s="18"/><row r="226" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A226" s="18"/><row r="227" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A227" s="18"/><row r="228" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A228" s="18"/><row r="229" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A229" s="18"/><row r="230" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A230" s="18"/><row r="231" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A231" s="18"/><row r="232" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A232" s="18"/><row r="233" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A233" s="18"/><row r="234" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A234" s="18"/><row r="235" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A235" s="18"/><row r="236" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A236" s="18"/><row r="237" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A237" s="18"/><row r="238" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A238" s="18"/><row r="239" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A239" s="18"/><row r="240" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A240" s="18"/><row r="241" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A241" s="18"/><row r="242" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A242" s="18"/><row r="243" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A243" s="18"/><row r="244" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A244" s="18"/><row r="245" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A245" s="18"/><row r="246" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A246" s="18"/><row r="247" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A247" s="18"/><row r="248" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A248" s="18"/><row r="249" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A249" s="18"/><row r="250" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A250" s="18"/><row r="251" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A251" s="18"/><row r="252" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A252" s="18"/><row r="253" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A253" s="18"/><row r="254" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A254" s="18"/><row r="255" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A255" s="18"/><row r="256" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A256" s="18"/><row r="257" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A257" s="18"/><row r="258" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A258" s="18"/><row r="259" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A259" s="18"/><row r="260" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A260" s="18"/><row r="261" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A261" s="18"/><row r="262" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A262" s="18"/><row r="263" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A263" s="18"/><row r="264" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A264" s="18"/><row r="265" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A265" s="18"/><row r="266" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A266" s="18"/><row r="267" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A267" s="18"/><row r="268" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A268" s="18"/><row r="269" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A269" s="18"/><row r="270" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A270" s="18"/><row r="271" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A271" s="18"/><row r="272" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A272" s="18"/><row r="273" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A273" s="18"/><row r="274" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A274" s="18"/><row r="275" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A275" s="18"/><row r="276" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A276" s="18"/><row r="277" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A277" s="18"/><row r="278" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A278" s="18"/><row r="279" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A279" s="18"/><row r="280" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A280" s="18"/><row r="281" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A281" s="18"/><row r="282" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A282" s="18"/><row r="283" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A283" s="18"/><row r="284" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A284" s="18"/><row r="285" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A285" s="18"/><row r="286" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A286" s="18"/><row r="287" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A287" s="18"/><row r="288" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A288" s="18"/><row r="289" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A289" s="18"/><row r="290" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A290" s="18"/><row r="291" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A291" s="18"/><row r="292" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A292" s="18"/><row r="293" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A293" s="18"/><row r="294" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A294" s="18"/><row r="295" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A295" s="18"/><row r="296" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A296" s="18"/><row r="297" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A297" s="18"/><row r="298" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A298" s="18"/><row r="299" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A299" s="18"/><row r="300" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A300" s="18"/><row r="301" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A301" s="18"/></sheetData><dataValidations count="4"><dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C3:C301" type="list"><formula1>_listas!$A$1:$A$6</formula1><formula2>0</formula2></dataValidation><dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E3:E301" type="list"><formula1>_listas!$B$1:$B$9</formula1><formula2>0</formula2></dataValidation><dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L3:L301" type="list"><formula1>_listas!$C$1:$C$3</formula1><formula2>0</formula2></dataValidation><dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J3:J301" type="list"><formula1>_listas!$D$1:$D$3</formula1><formula2>0</formula2></dataValidation></dataValidations><printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/><pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/><pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/><headerFooter differentFirst="false" differentOddEven="false"><oddHeader></oddHeader><oddFooter></oddFooter></headerFooter></worksheet>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:R301"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="16" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="40"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="K1" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="L1" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="M1" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="N1" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="O1" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="P1" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="Q1" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="R1" s="6" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>Modelo A</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="G2" s="8" t="n">
+        <v>200000</v>
+      </c>
+      <c r="H2" s="8" t="n">
+        <v>260000</v>
+      </c>
+      <c r="I2" s="9" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J2" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="K2" s="7" t="n">
+        <v>90</v>
+      </c>
+      <c r="L2" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="M2" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="N2" s="10" t="n">
+        <f aca="false">IFERROR(H2-G2,"")</f>
+        <v>60000</v>
+      </c>
+      <c r="O2" s="11" t="n">
+        <f aca="false">IFERROR(N2/H2,"")</f>
+        <v>0.230769230769231</v>
+      </c>
+      <c r="P2" s="10" t="n">
+        <f aca="false">IFERROR(SUMIF(cobranza!$B$3:$B$1000,A2,cobranza!$D$3:$D$1000),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q2" s="10" t="n">
+        <f aca="false">IFERROR(H2-P2,"")</f>
+        <v>260000</v>
+      </c>
+      <c r="R2" s="12" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="18"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="18"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="18"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="18"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="18"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="18"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="18"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="18"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="18"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="18"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="18"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="18"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="18"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="18"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="18"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="18"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="18"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="18"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="18"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="18"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="18"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="18"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="18"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="18"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="18"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="18"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="18"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="18"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="18"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="18"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="18"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="18"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="18"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="18"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="18"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="18"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="18"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="18"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="18"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="18"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="18"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="18"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="18"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="18"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="18"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="18"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="18"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="18"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="18"/>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="18"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="18"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="18"/>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="18"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="18"/>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="18"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="18"/>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="18"/>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="18"/>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="18"/>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="18"/>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="18"/>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="18"/>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="18"/>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="18"/>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="18"/>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="18"/>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="18"/>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="18"/>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="18"/>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="18"/>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="18"/>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="18"/>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="18"/>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="18"/>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="18"/>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="18"/>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="18"/>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="18"/>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="18"/>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="18"/>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="18"/>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="18"/>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="18"/>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="18"/>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="18"/>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="18"/>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="18"/>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="18"/>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="18"/>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="18"/>
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="18"/>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="18"/>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="18"/>
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="18"/>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="18"/>
+    </row>
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="18"/>
+    </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="18"/>
+    </row>
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="18"/>
+    </row>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="18"/>
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="18"/>
+    </row>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="18"/>
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="18"/>
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="18"/>
+    </row>
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="18"/>
+    </row>
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="18"/>
+    </row>
+    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="18"/>
+    </row>
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="18"/>
+    </row>
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="18"/>
+    </row>
+    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="18"/>
+    </row>
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="18"/>
+    </row>
+    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="18"/>
+    </row>
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="18"/>
+    </row>
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="18"/>
+    </row>
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="18"/>
+    </row>
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="18"/>
+    </row>
+    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="18"/>
+    </row>
+    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="18"/>
+    </row>
+    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="18"/>
+    </row>
+    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A121" s="18"/>
+    </row>
+    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A122" s="18"/>
+    </row>
+    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A123" s="18"/>
+    </row>
+    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A124" s="18"/>
+    </row>
+    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A125" s="18"/>
+    </row>
+    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A126" s="18"/>
+    </row>
+    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A127" s="18"/>
+    </row>
+    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A128" s="18"/>
+    </row>
+    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A129" s="18"/>
+    </row>
+    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A130" s="18"/>
+    </row>
+    <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A131" s="18"/>
+    </row>
+    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A132" s="18"/>
+    </row>
+    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A133" s="18"/>
+    </row>
+    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A134" s="18"/>
+    </row>
+    <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A135" s="18"/>
+    </row>
+    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A136" s="18"/>
+    </row>
+    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A137" s="18"/>
+    </row>
+    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A138" s="18"/>
+    </row>
+    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A139" s="18"/>
+    </row>
+    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A140" s="18"/>
+    </row>
+    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A141" s="18"/>
+    </row>
+    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A142" s="18"/>
+    </row>
+    <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A143" s="18"/>
+    </row>
+    <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A144" s="18"/>
+    </row>
+    <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A145" s="18"/>
+    </row>
+    <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A146" s="18"/>
+    </row>
+    <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A147" s="18"/>
+    </row>
+    <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A148" s="18"/>
+    </row>
+    <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A149" s="18"/>
+    </row>
+    <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A150" s="18"/>
+    </row>
+    <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A151" s="18"/>
+    </row>
+    <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A152" s="18"/>
+    </row>
+    <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A153" s="18"/>
+    </row>
+    <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A154" s="18"/>
+    </row>
+    <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A155" s="18"/>
+    </row>
+    <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A156" s="18"/>
+    </row>
+    <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A157" s="18"/>
+    </row>
+    <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A158" s="18"/>
+    </row>
+    <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A159" s="18"/>
+    </row>
+    <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A160" s="18"/>
+    </row>
+    <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A161" s="18"/>
+    </row>
+    <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A162" s="18"/>
+    </row>
+    <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A163" s="18"/>
+    </row>
+    <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A164" s="18"/>
+    </row>
+    <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A165" s="18"/>
+    </row>
+    <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A166" s="18"/>
+    </row>
+    <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A167" s="18"/>
+    </row>
+    <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A168" s="18"/>
+    </row>
+    <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A169" s="18"/>
+    </row>
+    <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A170" s="18"/>
+    </row>
+    <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A171" s="18"/>
+    </row>
+    <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A172" s="18"/>
+    </row>
+    <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A173" s="18"/>
+    </row>
+    <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A174" s="18"/>
+    </row>
+    <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A175" s="18"/>
+    </row>
+    <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A176" s="18"/>
+    </row>
+    <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A177" s="18"/>
+    </row>
+    <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A178" s="18"/>
+    </row>
+    <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A179" s="18"/>
+    </row>
+    <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A180" s="18"/>
+    </row>
+    <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A181" s="18"/>
+    </row>
+    <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A182" s="18"/>
+    </row>
+    <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A183" s="18"/>
+    </row>
+    <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A184" s="18"/>
+    </row>
+    <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A185" s="18"/>
+    </row>
+    <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A186" s="18"/>
+    </row>
+    <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A187" s="18"/>
+    </row>
+    <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A188" s="18"/>
+    </row>
+    <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A189" s="18"/>
+    </row>
+    <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A190" s="18"/>
+    </row>
+    <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A191" s="18"/>
+    </row>
+    <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A192" s="18"/>
+    </row>
+    <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A193" s="18"/>
+    </row>
+    <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A194" s="18"/>
+    </row>
+    <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A195" s="18"/>
+    </row>
+    <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A196" s="18"/>
+    </row>
+    <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A197" s="18"/>
+    </row>
+    <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A198" s="18"/>
+    </row>
+    <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A199" s="18"/>
+    </row>
+    <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A200" s="18"/>
+    </row>
+    <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A201" s="18"/>
+    </row>
+    <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A202" s="18"/>
+    </row>
+    <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A203" s="18"/>
+    </row>
+    <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A204" s="18"/>
+    </row>
+    <row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A205" s="18"/>
+    </row>
+    <row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A206" s="18"/>
+    </row>
+    <row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A207" s="18"/>
+    </row>
+    <row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A208" s="18"/>
+    </row>
+    <row r="209" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A209" s="18"/>
+    </row>
+    <row r="210" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A210" s="18"/>
+    </row>
+    <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A211" s="18"/>
+    </row>
+    <row r="212" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A212" s="18"/>
+    </row>
+    <row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A213" s="18"/>
+    </row>
+    <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A214" s="18"/>
+    </row>
+    <row r="215" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A215" s="18"/>
+    </row>
+    <row r="216" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A216" s="18"/>
+    </row>
+    <row r="217" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A217" s="18"/>
+    </row>
+    <row r="218" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A218" s="18"/>
+    </row>
+    <row r="219" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A219" s="18"/>
+    </row>
+    <row r="220" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A220" s="18"/>
+    </row>
+    <row r="221" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A221" s="18"/>
+    </row>
+    <row r="222" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A222" s="18"/>
+    </row>
+    <row r="223" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A223" s="18"/>
+    </row>
+    <row r="224" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A224" s="18"/>
+    </row>
+    <row r="225" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A225" s="18"/>
+    </row>
+    <row r="226" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A226" s="18"/>
+    </row>
+    <row r="227" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A227" s="18"/>
+    </row>
+    <row r="228" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A228" s="18"/>
+    </row>
+    <row r="229" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A229" s="18"/>
+    </row>
+    <row r="230" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A230" s="18"/>
+    </row>
+    <row r="231" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A231" s="18"/>
+    </row>
+    <row r="232" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A232" s="18"/>
+    </row>
+    <row r="233" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A233" s="18"/>
+    </row>
+    <row r="234" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A234" s="18"/>
+    </row>
+    <row r="235" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A235" s="18"/>
+    </row>
+    <row r="236" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A236" s="18"/>
+    </row>
+    <row r="237" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A237" s="18"/>
+    </row>
+    <row r="238" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A238" s="18"/>
+    </row>
+    <row r="239" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A239" s="18"/>
+    </row>
+    <row r="240" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A240" s="18"/>
+    </row>
+    <row r="241" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A241" s="18"/>
+    </row>
+    <row r="242" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A242" s="18"/>
+    </row>
+    <row r="243" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A243" s="18"/>
+    </row>
+    <row r="244" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A244" s="18"/>
+    </row>
+    <row r="245" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A245" s="18"/>
+    </row>
+    <row r="246" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A246" s="18"/>
+    </row>
+    <row r="247" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A247" s="18"/>
+    </row>
+    <row r="248" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A248" s="18"/>
+    </row>
+    <row r="249" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A249" s="18"/>
+    </row>
+    <row r="250" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A250" s="18"/>
+    </row>
+    <row r="251" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A251" s="18"/>
+    </row>
+    <row r="252" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A252" s="18"/>
+    </row>
+    <row r="253" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A253" s="18"/>
+    </row>
+    <row r="254" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A254" s="18"/>
+    </row>
+    <row r="255" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A255" s="18"/>
+    </row>
+    <row r="256" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A256" s="18"/>
+    </row>
+    <row r="257" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A257" s="18"/>
+    </row>
+    <row r="258" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A258" s="18"/>
+    </row>
+    <row r="259" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A259" s="18"/>
+    </row>
+    <row r="260" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A260" s="18"/>
+    </row>
+    <row r="261" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A261" s="18"/>
+    </row>
+    <row r="262" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A262" s="18"/>
+    </row>
+    <row r="263" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A263" s="18"/>
+    </row>
+    <row r="264" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A264" s="18"/>
+    </row>
+    <row r="265" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A265" s="18"/>
+    </row>
+    <row r="266" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A266" s="18"/>
+    </row>
+    <row r="267" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A267" s="18"/>
+    </row>
+    <row r="268" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A268" s="18"/>
+    </row>
+    <row r="269" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A269" s="18"/>
+    </row>
+    <row r="270" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A270" s="18"/>
+    </row>
+    <row r="271" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A271" s="18"/>
+    </row>
+    <row r="272" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A272" s="18"/>
+    </row>
+    <row r="273" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A273" s="18"/>
+    </row>
+    <row r="274" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A274" s="18"/>
+    </row>
+    <row r="275" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A275" s="18"/>
+    </row>
+    <row r="276" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A276" s="18"/>
+    </row>
+    <row r="277" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A277" s="18"/>
+    </row>
+    <row r="278" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A278" s="18"/>
+    </row>
+    <row r="279" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A279" s="18"/>
+    </row>
+    <row r="280" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A280" s="18"/>
+    </row>
+    <row r="281" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A281" s="18"/>
+    </row>
+    <row r="282" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A282" s="18"/>
+    </row>
+    <row r="283" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A283" s="18"/>
+    </row>
+    <row r="284" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A284" s="18"/>
+    </row>
+    <row r="285" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A285" s="18"/>
+    </row>
+    <row r="286" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A286" s="18"/>
+    </row>
+    <row r="287" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A287" s="18"/>
+    </row>
+    <row r="288" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A288" s="18"/>
+    </row>
+    <row r="289" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A289" s="18"/>
+    </row>
+    <row r="290" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A290" s="18"/>
+    </row>
+    <row r="291" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A291" s="18"/>
+    </row>
+    <row r="292" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A292" s="18"/>
+    </row>
+    <row r="293" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A293" s="18"/>
+    </row>
+    <row r="294" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A294" s="18"/>
+    </row>
+    <row r="295" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A295" s="18"/>
+    </row>
+    <row r="296" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A296" s="18"/>
+    </row>
+    <row r="297" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A297" s="18"/>
+    </row>
+    <row r="298" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A298" s="18"/>
+    </row>
+    <row r="299" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A299" s="18"/>
+    </row>
+    <row r="300" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A300" s="18"/>
+    </row>
+    <row r="301" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A301" s="18"/>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C3:C301" type="list">
+      <formula1>_listas!$A$1:$A$6</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L3:L301" type="list">
+      <formula1>_listas!$B$1:$B$3</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J3:J301" type="list">
+      <formula1>_listas!$C$1:$C$3</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="UTF-8" standalone="yes"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006"><sheetPr filterMode="false"><pageSetUpPr fitToPage="false"/></sheetPr><dimension ref="A1:G501"/><sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"></sheetFormatPr><cols><col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="12"/><col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/><col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="16"/><col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="34"/><col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="46"/></cols><sheetData><row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"><c r="A1" s="6" t="s"><v>165</v></c><c r="B1" s="6" t="s"><v>166</v></c><c r="C1" s="6" t="s"><v>167</v></c><c r="D1" s="6" t="s"><v>168</v></c><c r="E1" s="6" t="s"><v>169</v></c><c r="F1" s="6" t="s"><v>170</v></c><c r="G1" s="6" t="s"><v>100</v></c></row><row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A2" s="22" t="s"><v>171</v></c><c r="B2" s="22" t="s"><v>101</v></c><c r="C2" s="22" t="s"><v>172</v></c><c r="D2" s="23" t="n"><v>100000</v></c><c r="E2" s="22" t="s"><v>57</v></c><c r="F2" s="22" t="s"><v>103</v></c><c r="G2" s="22" t="s"><v>106</v></c></row><row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A3" s="13"/><row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A4" s="13"/><row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A5" s="13"/><row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A6" s="13"/><row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A7" s="13"/><row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A8" s="13"/><row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A9" s="13"/><row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A10" s="13"/><row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A11" s="13"/><row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A12" s="13"/><row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A13" s="13"/><row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A14" s="13"/><row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A15" s="13"/><row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A16" s="13"/><row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A17" s="13"/><row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A18" s="13"/><row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A19" s="13"/><row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A20" s="13"/><row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A21" s="13"/><row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A22" s="13"/><row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A23" s="13"/><row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A24" s="13"/><row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A25" s="13"/><row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A26" s="13"/><row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A27" s="13"/><row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A28" s="13"/><row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A29" s="13"/><row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A30" s="13"/><row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A31" s="13"/><row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A32" s="13"/><row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A33" s="13"/><row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A34" s="13"/><row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A35" s="13"/><row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A36" s="13"/><row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A37" s="13"/><row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A38" s="13"/><row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A39" s="13"/><row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A40" s="13"/><row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A41" s="13"/><row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A42" s="13"/><row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A43" s="13"/><row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A44" s="13"/><row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A45" s="13"/><row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A46" s="13"/><row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A47" s="13"/><row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A48" s="13"/><row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A49" s="13"/><row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A50" s="13"/><row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A51" s="13"/><row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A52" s="13"/><row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A53" s="13"/><row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A54" s="13"/><row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A55" s="13"/><row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A56" s="13"/><row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A57" s="13"/><row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A58" s="13"/><row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A59" s="13"/><row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A60" s="13"/><row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A61" s="13"/><row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A62" s="13"/><row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A63" s="13"/><row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A64" s="13"/><row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A65" s="13"/><row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A66" s="13"/><row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A67" s="13"/><row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A68" s="13"/><row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A69" s="13"/><row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A70" s="13"/><row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A71" s="13"/><row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A72" s="13"/><row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A73" s="13"/><row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A74" s="13"/><row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A75" s="13"/><row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A76" s="13"/><row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A77" s="13"/><row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A78" s="13"/><row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A79" s="13"/><row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A80" s="13"/><row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A81" s="13"/><row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A82" s="13"/><row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A83" s="13"/><row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A84" s="13"/><row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A85" s="13"/><row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A86" s="13"/><row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A87" s="13"/><row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A88" s="13"/><row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A89" s="13"/><row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A90" s="13"/><row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A91" s="13"/><row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A92" s="13"/><row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A93" s="13"/><row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A94" s="13"/><row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A95" s="13"/><row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A96" s="13"/><row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A97" s="13"/><row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A98" s="13"/><row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A99" s="13"/><row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A100" s="13"/><row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A101" s="13"/><row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A102" s="13"/><row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A103" s="13"/><row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A104" s="13"/><row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A105" s="13"/><row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A106" s="13"/><row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A107" s="13"/><row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A108" s="13"/><row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A109" s="13"/><row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A110" s="13"/><row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A111" s="13"/><row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A112" s="13"/><row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A113" s="13"/><row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A114" s="13"/><row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A115" s="13"/><row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A116" s="13"/><row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A117" s="13"/><row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A118" s="13"/><row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A119" s="13"/><row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A120" s="13"/><row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A121" s="13"/><row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A122" s="13"/><row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A123" s="13"/><row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A124" s="13"/><row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A125" s="13"/><row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A126" s="13"/><row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A127" s="13"/><row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A128" s="13"/><row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A129" s="13"/><row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A130" s="13"/><row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A131" s="13"/><row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A132" s="13"/><row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A133" s="13"/><row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A134" s="13"/><row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A135" s="13"/><row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A136" s="13"/><row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A137" s="13"/><row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A138" s="13"/><row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A139" s="13"/><row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A140" s="13"/><row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A141" s="13"/><row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A142" s="13"/><row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A143" s="13"/><row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A144" s="13"/><row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A145" s="13"/><row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A146" s="13"/><row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A147" s="13"/><row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A148" s="13"/><row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A149" s="13"/><row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A150" s="13"/><row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A151" s="13"/><row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A152" s="13"/><row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A153" s="13"/><row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A154" s="13"/><row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A155" s="13"/><row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A156" s="13"/><row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A157" s="13"/><row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A158" s="13"/><row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A159" s="13"/><row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A160" s="13"/><row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A161" s="13"/><row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A162" s="13"/><row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A163" s="13"/><row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A164" s="13"/><row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A165" s="13"/><row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A166" s="13"/><row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A167" s="13"/><row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A168" s="13"/><row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A169" s="13"/><row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A170" s="13"/><row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A171" s="13"/><row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A172" s="13"/><row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A173" s="13"/><row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A174" s="13"/><row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A175" s="13"/><row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A176" s="13"/><row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A177" s="13"/><row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A178" s="13"/><row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A179" s="13"/><row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A180" s="13"/><row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A181" s="13"/><row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A182" s="13"/><row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A183" s="13"/><row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A184" s="13"/><row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A185" s="13"/><row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A186" s="13"/><row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A187" s="13"/><row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A188" s="13"/><row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A189" s="13"/><row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A190" s="13"/><row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A191" s="13"/><row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A192" s="13"/><row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A193" s="13"/><row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A194" s="13"/><row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A195" s="13"/><row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A196" s="13"/><row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A197" s="13"/><row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A198" s="13"/><row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A199" s="13"/><row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A200" s="13"/><row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A201" s="13"/><row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A202" s="13"/><row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A203" s="13"/><row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A204" s="13"/><row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A205" s="13"/><row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A206" s="13"/><row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A207" s="13"/><row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A208" s="13"/><row r="209" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A209" s="13"/><row r="210" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A210" s="13"/><row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A211" s="13"/><row r="212" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A212" s="13"/><row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A213" s="13"/><row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A214" s="13"/><row r="215" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A215" s="13"/><row r="216" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A216" s="13"/><row r="217" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A217" s="13"/><row r="218" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A218" s="13"/><row r="219" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A219" s="13"/><row r="220" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A220" s="13"/><row r="221" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A221" s="13"/><row r="222" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A222" s="13"/><row r="223" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A223" s="13"/><row r="224" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A224" s="13"/><row r="225" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A225" s="13"/><row r="226" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A226" s="13"/><row r="227" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A227" s="13"/><row r="228" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A228" s="13"/><row r="229" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A229" s="13"/><row r="230" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A230" s="13"/><row r="231" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A231" s="13"/><row r="232" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A232" s="13"/><row r="233" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A233" s="13"/><row r="234" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A234" s="13"/><row r="235" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A235" s="13"/><row r="236" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A236" s="13"/><row r="237" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A237" s="13"/><row r="238" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A238" s="13"/><row r="239" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A239" s="13"/><row r="240" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A240" s="13"/><row r="241" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A241" s="13"/><row r="242" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A242" s="13"/><row r="243" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A243" s="13"/><row r="244" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A244" s="13"/><row r="245" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A245" s="13"/><row r="246" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A246" s="13"/><row r="247" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A247" s="13"/><row r="248" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A248" s="13"/><row r="249" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A249" s="13"/><row r="250" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A250" s="13"/><row r="251" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A251" s="13"/><row r="252" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A252" s="13"/><row r="253" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A253" s="13"/><row r="254" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A254" s="13"/><row r="255" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A255" s="13"/><row r="256" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A256" s="13"/><row r="257" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A257" s="13"/><row r="258" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A258" s="13"/><row r="259" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A259" s="13"/><row r="260" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A260" s="13"/><row r="261" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A261" s="13"/><row r="262" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A262" s="13"/><row r="263" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A263" s="13"/><row r="264" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A264" s="13"/><row r="265" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A265" s="13"/><row r="266" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A266" s="13"/><row r="267" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A267" s="13"/><row r="268" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A268" s="13"/><row r="269" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A269" s="13"/><row r="270" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A270" s="13"/><row r="271" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A271" s="13"/><row r="272" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A272" s="13"/><row r="273" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A273" s="13"/><row r="274" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A274" s="13"/><row r="275" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A275" s="13"/><row r="276" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A276" s="13"/><row r="277" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A277" s="13"/><row r="278" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A278" s="13"/><row r="279" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A279" s="13"/><row r="280" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A280" s="13"/><row r="281" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A281" s="13"/><row r="282" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A282" s="13"/><row r="283" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A283" s="13"/><row r="284" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A284" s="13"/><row r="285" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A285" s="13"/><row r="286" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A286" s="13"/><row r="287" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A287" s="13"/><row r="288" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A288" s="13"/><row r="289" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A289" s="13"/><row r="290" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A290" s="13"/><row r="291" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A291" s="13"/><row r="292" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A292" s="13"/><row r="293" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A293" s="13"/><row r="294" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A294" s="13"/><row r="295" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A295" s="13"/><row r="296" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A296" s="13"/><row r="297" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A297" s="13"/><row r="298" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A298" s="13"/><row r="299" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A299" s="13"/><row r="300" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A300" s="13"/><row r="301" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A301" s="13"/><row r="302" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A302" s="13"/><row r="303" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A303" s="13"/><row r="304" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A304" s="13"/><row r="305" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A305" s="13"/><row r="306" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A306" s="13"/><row r="307" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A307" s="13"/><row r="308" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A308" s="13"/><row r="309" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A309" s="13"/><row r="310" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A310" s="13"/><row r="311" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A311" s="13"/><row r="312" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A312" s="13"/><row r="313" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A313" s="13"/><row r="314" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A314" s="13"/><row r="315" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A315" s="13"/><row r="316" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A316" s="13"/><row r="317" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A317" s="13"/><row r="318" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A318" s="13"/><row r="319" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A319" s="13"/><row r="320" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A320" s="13"/><row r="321" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A321" s="13"/><row r="322" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A322" s="13"/><row r="323" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A323" s="13"/><row r="324" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A324" s="13"/><row r="325" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A325" s="13"/><row r="326" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A326" s="13"/><row r="327" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A327" s="13"/><row r="328" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A328" s="13"/><row r="329" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A329" s="13"/><row r="330" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A330" s="13"/><row r="331" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A331" s="13"/><row r="332" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A332" s="13"/><row r="333" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A333" s="13"/><row r="334" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A334" s="13"/><row r="335" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A335" s="13"/><row r="336" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A336" s="13"/><row r="337" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A337" s="13"/><row r="338" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A338" s="13"/><row r="339" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A339" s="13"/><row r="340" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A340" s="13"/><row r="341" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A341" s="13"/><row r="342" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A342" s="13"/><row r="343" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A343" s="13"/><row r="344" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A344" s="13"/><row r="345" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A345" s="13"/><row r="346" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A346" s="13"/><row r="347" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A347" s="13"/><row r="348" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A348" s="13"/><row r="349" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A349" s="13"/><row r="350" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A350" s="13"/><row r="351" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A351" s="13"/><row r="352" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A352" s="13"/><row r="353" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A353" s="13"/><row r="354" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A354" s="13"/><row r="355" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A355" s="13"/><row r="356" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A356" s="13"/><row r="357" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A357" s="13"/><row r="358" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A358" s="13"/><row r="359" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A359" s="13"/><row r="360" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A360" s="13"/><row r="361" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A361" s="13"/><row r="362" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A362" s="13"/><row r="363" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A363" s="13"/><row r="364" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A364" s="13"/><row r="365" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A365" s="13"/><row r="366" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A366" s="13"/><row r="367" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A367" s="13"/><row r="368" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A368" s="13"/><row r="369" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A369" s="13"/><row r="370" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A370" s="13"/><row r="371" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A371" s="13"/><row r="372" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A372" s="13"/><row r="373" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A373" s="13"/><row r="374" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A374" s="13"/><row r="375" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A375" s="13"/><row r="376" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A376" s="13"/><row r="377" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A377" s="13"/><row r="378" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A378" s="13"/><row r="379" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A379" s="13"/><row r="380" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A380" s="13"/><row r="381" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A381" s="13"/><row r="382" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A382" s="13"/><row r="383" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A383" s="13"/><row r="384" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A384" s="13"/><row r="385" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A385" s="13"/><row r="386" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A386" s="13"/><row r="387" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A387" s="13"/><row r="388" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A388" s="13"/><row r="389" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A389" s="13"/><row r="390" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A390" s="13"/><row r="391" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A391" s="13"/><row r="392" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A392" s="13"/><row r="393" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A393" s="13"/><row r="394" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A394" s="13"/><row r="395" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A395" s="13"/><row r="396" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A396" s="13"/><row r="397" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A397" s="13"/><row r="398" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A398" s="13"/><row r="399" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A399" s="13"/><row r="400" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A400" s="13"/><row r="401" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A401" s="13"/><row r="402" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A402" s="13"/><row r="403" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A403" s="13"/><row r="404" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A404" s="13"/><row r="405" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A405" s="13"/><row r="406" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A406" s="13"/><row r="407" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A407" s="13"/><row r="408" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A408" s="13"/><row r="409" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A409" s="13"/><row r="410" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A410" s="13"/><row r="411" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A411" s="13"/><row r="412" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A412" s="13"/><row r="413" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A413" s="13"/><row r="414" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A414" s="13"/><row r="415" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A415" s="13"/><row r="416" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A416" s="13"/><row r="417" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A417" s="13"/><row r="418" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A418" s="13"/><row r="419" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A419" s="13"/><row r="420" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A420" s="13"/><row r="421" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A421" s="13"/><row r="422" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A422" s="13"/><row r="423" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A423" s="13"/><row r="424" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A424" s="13"/><row r="425" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A425" s="13"/><row r="426" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A426" s="13"/><row r="427" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A427" s="13"/><row r="428" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A428" s="13"/><row r="429" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A429" s="13"/><row r="430" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A430" s="13"/><row r="431" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A431" s="13"/><row r="432" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A432" s="13"/><row r="433" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A433" s="13"/><row r="434" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A434" s="13"/><row r="435" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A435" s="13"/><row r="436" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A436" s="13"/><row r="437" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A437" s="13"/><row r="438" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A438" s="13"/><row r="439" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A439" s="13"/><row r="440" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A440" s="13"/><row r="441" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A441" s="13"/><row r="442" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A442" s="13"/><row r="443" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A443" s="13"/><row r="444" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A444" s="13"/><row r="445" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A445" s="13"/><row r="446" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A446" s="13"/><row r="447" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A447" s="13"/><row r="448" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A448" s="13"/><row r="449" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A449" s="13"/><row r="450" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A450" s="13"/><row r="451" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A451" s="13"/><row r="452" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A452" s="13"/><row r="453" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A453" s="13"/><row r="454" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A454" s="13"/><row r="455" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A455" s="13"/><row r="456" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A456" s="13"/><row r="457" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A457" s="13"/><row r="458" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A458" s="13"/><row r="459" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A459" s="13"/><row r="460" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A460" s="13"/><row r="461" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A461" s="13"/><row r="462" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A462" s="13"/><row r="463" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A463" s="13"/><row r="464" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A464" s="13"/><row r="465" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A465" s="13"/><row r="466" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A466" s="13"/><row r="467" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A467" s="13"/><row r="468" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A468" s="13"/><row r="469" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A469" s="13"/><row r="470" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A470" s="13"/><row r="471" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A471" s="13"/><row r="472" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A472" s="13"/><row r="473" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A473" s="13"/><row r="474" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A474" s="13"/><row r="475" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A475" s="13"/><row r="476" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A476" s="13"/><row r="477" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A477" s="13"/><row r="478" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A478" s="13"/><row r="479" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A479" s="13"/><row r="480" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A480" s="13"/><row r="481" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A481" s="13"/><row r="482" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A482" s="13"/><row r="483" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A483" s="13"/><row r="484" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A484" s="13"/><row r="485" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A485" s="13"/><row r="486" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A486" s="13"/><row r="487" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A487" s="13"/><row r="488" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A488" s="13"/><row r="489" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A489" s="13"/><row r="490" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A490" s="13"/><row r="491" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A491" s="13"/><row r="492" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A492" s="13"/><row r="493" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A493" s="13"/><row r="494" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A494" s="13"/><row r="495" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A495" s="13"/><row r="496" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A496" s="13"/><row r="497" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A497" s="13"/><row r="498" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A498" s="13"/><row r="499" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A499" s="13"/><row r="500" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A500" s="13"/><row r="501" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A501" s="13"/></sheetData><dataValidations count="1"><dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E3:E501" type="list"><formula1>_listas!$G$1:$G$5</formula1><formula2>0</formula2></dataValidation></dataValidations><printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/><pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/><pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/><headerFooter differentFirst="false" differentOddEven="false"><oddHeader></oddHeader><oddFooter></oddFooter></headerFooter></worksheet>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:G501"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="46"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="22" t="s">
+        <v>171</v>
+      </c>
+      <c r="B2" s="22" t="s">
+        <v>101</v>
+      </c>
+      <c r="C2" s="22" t="s">
+        <v>172</v>
+      </c>
+      <c r="D2" s="23" t="n">
+        <v>100000</v>
+      </c>
+      <c r="E2" s="22" t="s">
+        <v>57</v>
+      </c>
+      <c r="F2" s="22" t="s">
+        <v>103</v>
+      </c>
+      <c r="G2" s="22" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="13"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="13"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="13"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="13"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="13"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="13"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="13"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="13"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="13"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="13"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="13"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="13"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="13"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="13"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="13"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="13"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="13"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="13"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="13"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="13"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="13"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="13"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="13"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="13"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="13"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="13"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="13"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="13"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="13"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="13"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="13"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="13"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="13"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="13"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="13"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="13"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="13"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="13"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="13"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="13"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="13"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="13"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="13"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="13"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="13"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="13"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="13"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="13"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="13"/>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="13"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="13"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="13"/>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="13"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="13"/>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="13"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="13"/>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="13"/>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="13"/>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="13"/>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="13"/>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="13"/>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="13"/>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="13"/>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="13"/>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="13"/>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="13"/>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="13"/>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="13"/>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="13"/>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="13"/>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="13"/>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="13"/>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="13"/>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="13"/>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="13"/>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="13"/>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="13"/>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="13"/>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="13"/>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="13"/>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="13"/>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="13"/>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="13"/>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="13"/>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="13"/>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="13"/>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="13"/>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="13"/>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="13"/>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="13"/>
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="13"/>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="13"/>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="13"/>
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="13"/>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="13"/>
+    </row>
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="13"/>
+    </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="13"/>
+    </row>
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="13"/>
+    </row>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="13"/>
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="13"/>
+    </row>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="13"/>
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="13"/>
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="13"/>
+    </row>
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="13"/>
+    </row>
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="13"/>
+    </row>
+    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="13"/>
+    </row>
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="13"/>
+    </row>
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="13"/>
+    </row>
+    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="13"/>
+    </row>
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="13"/>
+    </row>
+    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="13"/>
+    </row>
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="13"/>
+    </row>
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="13"/>
+    </row>
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="13"/>
+    </row>
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="13"/>
+    </row>
+    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="13"/>
+    </row>
+    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="13"/>
+    </row>
+    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="13"/>
+    </row>
+    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A121" s="13"/>
+    </row>
+    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A122" s="13"/>
+    </row>
+    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A123" s="13"/>
+    </row>
+    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A124" s="13"/>
+    </row>
+    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A125" s="13"/>
+    </row>
+    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A126" s="13"/>
+    </row>
+    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A127" s="13"/>
+    </row>
+    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A128" s="13"/>
+    </row>
+    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A129" s="13"/>
+    </row>
+    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A130" s="13"/>
+    </row>
+    <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A131" s="13"/>
+    </row>
+    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A132" s="13"/>
+    </row>
+    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A133" s="13"/>
+    </row>
+    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A134" s="13"/>
+    </row>
+    <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A135" s="13"/>
+    </row>
+    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A136" s="13"/>
+    </row>
+    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A137" s="13"/>
+    </row>
+    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A138" s="13"/>
+    </row>
+    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A139" s="13"/>
+    </row>
+    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A140" s="13"/>
+    </row>
+    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A141" s="13"/>
+    </row>
+    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A142" s="13"/>
+    </row>
+    <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A143" s="13"/>
+    </row>
+    <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A144" s="13"/>
+    </row>
+    <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A145" s="13"/>
+    </row>
+    <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A146" s="13"/>
+    </row>
+    <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A147" s="13"/>
+    </row>
+    <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A148" s="13"/>
+    </row>
+    <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A149" s="13"/>
+    </row>
+    <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A150" s="13"/>
+    </row>
+    <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A151" s="13"/>
+    </row>
+    <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A152" s="13"/>
+    </row>
+    <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A153" s="13"/>
+    </row>
+    <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A154" s="13"/>
+    </row>
+    <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A155" s="13"/>
+    </row>
+    <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A156" s="13"/>
+    </row>
+    <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A157" s="13"/>
+    </row>
+    <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A158" s="13"/>
+    </row>
+    <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A159" s="13"/>
+    </row>
+    <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A160" s="13"/>
+    </row>
+    <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A161" s="13"/>
+    </row>
+    <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A162" s="13"/>
+    </row>
+    <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A163" s="13"/>
+    </row>
+    <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A164" s="13"/>
+    </row>
+    <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A165" s="13"/>
+    </row>
+    <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A166" s="13"/>
+    </row>
+    <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A167" s="13"/>
+    </row>
+    <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A168" s="13"/>
+    </row>
+    <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A169" s="13"/>
+    </row>
+    <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A170" s="13"/>
+    </row>
+    <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A171" s="13"/>
+    </row>
+    <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A172" s="13"/>
+    </row>
+    <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A173" s="13"/>
+    </row>
+    <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A174" s="13"/>
+    </row>
+    <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A175" s="13"/>
+    </row>
+    <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A176" s="13"/>
+    </row>
+    <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A177" s="13"/>
+    </row>
+    <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A178" s="13"/>
+    </row>
+    <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A179" s="13"/>
+    </row>
+    <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A180" s="13"/>
+    </row>
+    <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A181" s="13"/>
+    </row>
+    <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A182" s="13"/>
+    </row>
+    <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A183" s="13"/>
+    </row>
+    <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A184" s="13"/>
+    </row>
+    <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A185" s="13"/>
+    </row>
+    <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A186" s="13"/>
+    </row>
+    <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A187" s="13"/>
+    </row>
+    <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A188" s="13"/>
+    </row>
+    <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A189" s="13"/>
+    </row>
+    <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A190" s="13"/>
+    </row>
+    <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A191" s="13"/>
+    </row>
+    <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A192" s="13"/>
+    </row>
+    <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A193" s="13"/>
+    </row>
+    <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A194" s="13"/>
+    </row>
+    <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A195" s="13"/>
+    </row>
+    <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A196" s="13"/>
+    </row>
+    <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A197" s="13"/>
+    </row>
+    <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A198" s="13"/>
+    </row>
+    <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A199" s="13"/>
+    </row>
+    <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A200" s="13"/>
+    </row>
+    <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A201" s="13"/>
+    </row>
+    <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A202" s="13"/>
+    </row>
+    <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A203" s="13"/>
+    </row>
+    <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A204" s="13"/>
+    </row>
+    <row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A205" s="13"/>
+    </row>
+    <row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A206" s="13"/>
+    </row>
+    <row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A207" s="13"/>
+    </row>
+    <row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A208" s="13"/>
+    </row>
+    <row r="209" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A209" s="13"/>
+    </row>
+    <row r="210" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A210" s="13"/>
+    </row>
+    <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A211" s="13"/>
+    </row>
+    <row r="212" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A212" s="13"/>
+    </row>
+    <row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A213" s="13"/>
+    </row>
+    <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A214" s="13"/>
+    </row>
+    <row r="215" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A215" s="13"/>
+    </row>
+    <row r="216" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A216" s="13"/>
+    </row>
+    <row r="217" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A217" s="13"/>
+    </row>
+    <row r="218" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A218" s="13"/>
+    </row>
+    <row r="219" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A219" s="13"/>
+    </row>
+    <row r="220" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A220" s="13"/>
+    </row>
+    <row r="221" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A221" s="13"/>
+    </row>
+    <row r="222" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A222" s="13"/>
+    </row>
+    <row r="223" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A223" s="13"/>
+    </row>
+    <row r="224" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A224" s="13"/>
+    </row>
+    <row r="225" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A225" s="13"/>
+    </row>
+    <row r="226" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A226" s="13"/>
+    </row>
+    <row r="227" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A227" s="13"/>
+    </row>
+    <row r="228" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A228" s="13"/>
+    </row>
+    <row r="229" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A229" s="13"/>
+    </row>
+    <row r="230" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A230" s="13"/>
+    </row>
+    <row r="231" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A231" s="13"/>
+    </row>
+    <row r="232" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A232" s="13"/>
+    </row>
+    <row r="233" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A233" s="13"/>
+    </row>
+    <row r="234" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A234" s="13"/>
+    </row>
+    <row r="235" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A235" s="13"/>
+    </row>
+    <row r="236" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A236" s="13"/>
+    </row>
+    <row r="237" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A237" s="13"/>
+    </row>
+    <row r="238" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A238" s="13"/>
+    </row>
+    <row r="239" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A239" s="13"/>
+    </row>
+    <row r="240" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A240" s="13"/>
+    </row>
+    <row r="241" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A241" s="13"/>
+    </row>
+    <row r="242" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A242" s="13"/>
+    </row>
+    <row r="243" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A243" s="13"/>
+    </row>
+    <row r="244" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A244" s="13"/>
+    </row>
+    <row r="245" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A245" s="13"/>
+    </row>
+    <row r="246" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A246" s="13"/>
+    </row>
+    <row r="247" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A247" s="13"/>
+    </row>
+    <row r="248" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A248" s="13"/>
+    </row>
+    <row r="249" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A249" s="13"/>
+    </row>
+    <row r="250" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A250" s="13"/>
+    </row>
+    <row r="251" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A251" s="13"/>
+    </row>
+    <row r="252" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A252" s="13"/>
+    </row>
+    <row r="253" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A253" s="13"/>
+    </row>
+    <row r="254" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A254" s="13"/>
+    </row>
+    <row r="255" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A255" s="13"/>
+    </row>
+    <row r="256" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A256" s="13"/>
+    </row>
+    <row r="257" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A257" s="13"/>
+    </row>
+    <row r="258" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A258" s="13"/>
+    </row>
+    <row r="259" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A259" s="13"/>
+    </row>
+    <row r="260" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A260" s="13"/>
+    </row>
+    <row r="261" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A261" s="13"/>
+    </row>
+    <row r="262" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A262" s="13"/>
+    </row>
+    <row r="263" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A263" s="13"/>
+    </row>
+    <row r="264" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A264" s="13"/>
+    </row>
+    <row r="265" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A265" s="13"/>
+    </row>
+    <row r="266" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A266" s="13"/>
+    </row>
+    <row r="267" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A267" s="13"/>
+    </row>
+    <row r="268" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A268" s="13"/>
+    </row>
+    <row r="269" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A269" s="13"/>
+    </row>
+    <row r="270" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A270" s="13"/>
+    </row>
+    <row r="271" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A271" s="13"/>
+    </row>
+    <row r="272" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A272" s="13"/>
+    </row>
+    <row r="273" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A273" s="13"/>
+    </row>
+    <row r="274" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A274" s="13"/>
+    </row>
+    <row r="275" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A275" s="13"/>
+    </row>
+    <row r="276" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A276" s="13"/>
+    </row>
+    <row r="277" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A277" s="13"/>
+    </row>
+    <row r="278" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A278" s="13"/>
+    </row>
+    <row r="279" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A279" s="13"/>
+    </row>
+    <row r="280" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A280" s="13"/>
+    </row>
+    <row r="281" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A281" s="13"/>
+    </row>
+    <row r="282" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A282" s="13"/>
+    </row>
+    <row r="283" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A283" s="13"/>
+    </row>
+    <row r="284" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A284" s="13"/>
+    </row>
+    <row r="285" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A285" s="13"/>
+    </row>
+    <row r="286" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A286" s="13"/>
+    </row>
+    <row r="287" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A287" s="13"/>
+    </row>
+    <row r="288" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A288" s="13"/>
+    </row>
+    <row r="289" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A289" s="13"/>
+    </row>
+    <row r="290" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A290" s="13"/>
+    </row>
+    <row r="291" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A291" s="13"/>
+    </row>
+    <row r="292" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A292" s="13"/>
+    </row>
+    <row r="293" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A293" s="13"/>
+    </row>
+    <row r="294" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A294" s="13"/>
+    </row>
+    <row r="295" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A295" s="13"/>
+    </row>
+    <row r="296" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A296" s="13"/>
+    </row>
+    <row r="297" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A297" s="13"/>
+    </row>
+    <row r="298" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A298" s="13"/>
+    </row>
+    <row r="299" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A299" s="13"/>
+    </row>
+    <row r="300" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A300" s="13"/>
+    </row>
+    <row r="301" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A301" s="13"/>
+    </row>
+    <row r="302" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A302" s="13"/>
+    </row>
+    <row r="303" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A303" s="13"/>
+    </row>
+    <row r="304" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A304" s="13"/>
+    </row>
+    <row r="305" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A305" s="13"/>
+    </row>
+    <row r="306" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A306" s="13"/>
+    </row>
+    <row r="307" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A307" s="13"/>
+    </row>
+    <row r="308" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A308" s="13"/>
+    </row>
+    <row r="309" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A309" s="13"/>
+    </row>
+    <row r="310" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A310" s="13"/>
+    </row>
+    <row r="311" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A311" s="13"/>
+    </row>
+    <row r="312" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A312" s="13"/>
+    </row>
+    <row r="313" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A313" s="13"/>
+    </row>
+    <row r="314" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A314" s="13"/>
+    </row>
+    <row r="315" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A315" s="13"/>
+    </row>
+    <row r="316" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A316" s="13"/>
+    </row>
+    <row r="317" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A317" s="13"/>
+    </row>
+    <row r="318" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A318" s="13"/>
+    </row>
+    <row r="319" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A319" s="13"/>
+    </row>
+    <row r="320" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A320" s="13"/>
+    </row>
+    <row r="321" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A321" s="13"/>
+    </row>
+    <row r="322" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A322" s="13"/>
+    </row>
+    <row r="323" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A323" s="13"/>
+    </row>
+    <row r="324" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A324" s="13"/>
+    </row>
+    <row r="325" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A325" s="13"/>
+    </row>
+    <row r="326" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A326" s="13"/>
+    </row>
+    <row r="327" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A327" s="13"/>
+    </row>
+    <row r="328" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A328" s="13"/>
+    </row>
+    <row r="329" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A329" s="13"/>
+    </row>
+    <row r="330" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A330" s="13"/>
+    </row>
+    <row r="331" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A331" s="13"/>
+    </row>
+    <row r="332" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A332" s="13"/>
+    </row>
+    <row r="333" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A333" s="13"/>
+    </row>
+    <row r="334" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A334" s="13"/>
+    </row>
+    <row r="335" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A335" s="13"/>
+    </row>
+    <row r="336" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A336" s="13"/>
+    </row>
+    <row r="337" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A337" s="13"/>
+    </row>
+    <row r="338" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A338" s="13"/>
+    </row>
+    <row r="339" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A339" s="13"/>
+    </row>
+    <row r="340" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A340" s="13"/>
+    </row>
+    <row r="341" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A341" s="13"/>
+    </row>
+    <row r="342" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A342" s="13"/>
+    </row>
+    <row r="343" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A343" s="13"/>
+    </row>
+    <row r="344" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A344" s="13"/>
+    </row>
+    <row r="345" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A345" s="13"/>
+    </row>
+    <row r="346" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A346" s="13"/>
+    </row>
+    <row r="347" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A347" s="13"/>
+    </row>
+    <row r="348" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A348" s="13"/>
+    </row>
+    <row r="349" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A349" s="13"/>
+    </row>
+    <row r="350" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A350" s="13"/>
+    </row>
+    <row r="351" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A351" s="13"/>
+    </row>
+    <row r="352" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A352" s="13"/>
+    </row>
+    <row r="353" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A353" s="13"/>
+    </row>
+    <row r="354" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A354" s="13"/>
+    </row>
+    <row r="355" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A355" s="13"/>
+    </row>
+    <row r="356" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A356" s="13"/>
+    </row>
+    <row r="357" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A357" s="13"/>
+    </row>
+    <row r="358" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A358" s="13"/>
+    </row>
+    <row r="359" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A359" s="13"/>
+    </row>
+    <row r="360" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A360" s="13"/>
+    </row>
+    <row r="361" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A361" s="13"/>
+    </row>
+    <row r="362" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A362" s="13"/>
+    </row>
+    <row r="363" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A363" s="13"/>
+    </row>
+    <row r="364" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A364" s="13"/>
+    </row>
+    <row r="365" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A365" s="13"/>
+    </row>
+    <row r="366" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A366" s="13"/>
+    </row>
+    <row r="367" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A367" s="13"/>
+    </row>
+    <row r="368" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A368" s="13"/>
+    </row>
+    <row r="369" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A369" s="13"/>
+    </row>
+    <row r="370" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A370" s="13"/>
+    </row>
+    <row r="371" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A371" s="13"/>
+    </row>
+    <row r="372" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A372" s="13"/>
+    </row>
+    <row r="373" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A373" s="13"/>
+    </row>
+    <row r="374" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A374" s="13"/>
+    </row>
+    <row r="375" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A375" s="13"/>
+    </row>
+    <row r="376" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A376" s="13"/>
+    </row>
+    <row r="377" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A377" s="13"/>
+    </row>
+    <row r="378" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A378" s="13"/>
+    </row>
+    <row r="379" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A379" s="13"/>
+    </row>
+    <row r="380" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A380" s="13"/>
+    </row>
+    <row r="381" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A381" s="13"/>
+    </row>
+    <row r="382" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A382" s="13"/>
+    </row>
+    <row r="383" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A383" s="13"/>
+    </row>
+    <row r="384" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A384" s="13"/>
+    </row>
+    <row r="385" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A385" s="13"/>
+    </row>
+    <row r="386" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A386" s="13"/>
+    </row>
+    <row r="387" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A387" s="13"/>
+    </row>
+    <row r="388" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A388" s="13"/>
+    </row>
+    <row r="389" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A389" s="13"/>
+    </row>
+    <row r="390" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A390" s="13"/>
+    </row>
+    <row r="391" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A391" s="13"/>
+    </row>
+    <row r="392" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A392" s="13"/>
+    </row>
+    <row r="393" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A393" s="13"/>
+    </row>
+    <row r="394" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A394" s="13"/>
+    </row>
+    <row r="395" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A395" s="13"/>
+    </row>
+    <row r="396" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A396" s="13"/>
+    </row>
+    <row r="397" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A397" s="13"/>
+    </row>
+    <row r="398" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A398" s="13"/>
+    </row>
+    <row r="399" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A399" s="13"/>
+    </row>
+    <row r="400" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A400" s="13"/>
+    </row>
+    <row r="401" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A401" s="13"/>
+    </row>
+    <row r="402" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A402" s="13"/>
+    </row>
+    <row r="403" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A403" s="13"/>
+    </row>
+    <row r="404" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A404" s="13"/>
+    </row>
+    <row r="405" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A405" s="13"/>
+    </row>
+    <row r="406" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A406" s="13"/>
+    </row>
+    <row r="407" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A407" s="13"/>
+    </row>
+    <row r="408" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A408" s="13"/>
+    </row>
+    <row r="409" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A409" s="13"/>
+    </row>
+    <row r="410" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A410" s="13"/>
+    </row>
+    <row r="411" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A411" s="13"/>
+    </row>
+    <row r="412" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A412" s="13"/>
+    </row>
+    <row r="413" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A413" s="13"/>
+    </row>
+    <row r="414" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A414" s="13"/>
+    </row>
+    <row r="415" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A415" s="13"/>
+    </row>
+    <row r="416" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A416" s="13"/>
+    </row>
+    <row r="417" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A417" s="13"/>
+    </row>
+    <row r="418" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A418" s="13"/>
+    </row>
+    <row r="419" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A419" s="13"/>
+    </row>
+    <row r="420" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A420" s="13"/>
+    </row>
+    <row r="421" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A421" s="13"/>
+    </row>
+    <row r="422" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A422" s="13"/>
+    </row>
+    <row r="423" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A423" s="13"/>
+    </row>
+    <row r="424" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A424" s="13"/>
+    </row>
+    <row r="425" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A425" s="13"/>
+    </row>
+    <row r="426" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A426" s="13"/>
+    </row>
+    <row r="427" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A427" s="13"/>
+    </row>
+    <row r="428" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A428" s="13"/>
+    </row>
+    <row r="429" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A429" s="13"/>
+    </row>
+    <row r="430" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A430" s="13"/>
+    </row>
+    <row r="431" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A431" s="13"/>
+    </row>
+    <row r="432" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A432" s="13"/>
+    </row>
+    <row r="433" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A433" s="13"/>
+    </row>
+    <row r="434" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A434" s="13"/>
+    </row>
+    <row r="435" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A435" s="13"/>
+    </row>
+    <row r="436" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A436" s="13"/>
+    </row>
+    <row r="437" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A437" s="13"/>
+    </row>
+    <row r="438" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A438" s="13"/>
+    </row>
+    <row r="439" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A439" s="13"/>
+    </row>
+    <row r="440" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A440" s="13"/>
+    </row>
+    <row r="441" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A441" s="13"/>
+    </row>
+    <row r="442" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A442" s="13"/>
+    </row>
+    <row r="443" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A443" s="13"/>
+    </row>
+    <row r="444" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A444" s="13"/>
+    </row>
+    <row r="445" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A445" s="13"/>
+    </row>
+    <row r="446" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A446" s="13"/>
+    </row>
+    <row r="447" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A447" s="13"/>
+    </row>
+    <row r="448" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A448" s="13"/>
+    </row>
+    <row r="449" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A449" s="13"/>
+    </row>
+    <row r="450" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A450" s="13"/>
+    </row>
+    <row r="451" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A451" s="13"/>
+    </row>
+    <row r="452" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A452" s="13"/>
+    </row>
+    <row r="453" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A453" s="13"/>
+    </row>
+    <row r="454" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A454" s="13"/>
+    </row>
+    <row r="455" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A455" s="13"/>
+    </row>
+    <row r="456" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A456" s="13"/>
+    </row>
+    <row r="457" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A457" s="13"/>
+    </row>
+    <row r="458" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A458" s="13"/>
+    </row>
+    <row r="459" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A459" s="13"/>
+    </row>
+    <row r="460" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A460" s="13"/>
+    </row>
+    <row r="461" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A461" s="13"/>
+    </row>
+    <row r="462" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A462" s="13"/>
+    </row>
+    <row r="463" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A463" s="13"/>
+    </row>
+    <row r="464" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A464" s="13"/>
+    </row>
+    <row r="465" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A465" s="13"/>
+    </row>
+    <row r="466" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A466" s="13"/>
+    </row>
+    <row r="467" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A467" s="13"/>
+    </row>
+    <row r="468" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A468" s="13"/>
+    </row>
+    <row r="469" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A469" s="13"/>
+    </row>
+    <row r="470" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A470" s="13"/>
+    </row>
+    <row r="471" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A471" s="13"/>
+    </row>
+    <row r="472" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A472" s="13"/>
+    </row>
+    <row r="473" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A473" s="13"/>
+    </row>
+    <row r="474" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A474" s="13"/>
+    </row>
+    <row r="475" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A475" s="13"/>
+    </row>
+    <row r="476" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A476" s="13"/>
+    </row>
+    <row r="477" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A477" s="13"/>
+    </row>
+    <row r="478" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A478" s="13"/>
+    </row>
+    <row r="479" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A479" s="13"/>
+    </row>
+    <row r="480" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A480" s="13"/>
+    </row>
+    <row r="481" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A481" s="13"/>
+    </row>
+    <row r="482" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A482" s="13"/>
+    </row>
+    <row r="483" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A483" s="13"/>
+    </row>
+    <row r="484" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A484" s="13"/>
+    </row>
+    <row r="485" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A485" s="13"/>
+    </row>
+    <row r="486" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A486" s="13"/>
+    </row>
+    <row r="487" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A487" s="13"/>
+    </row>
+    <row r="488" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A488" s="13"/>
+    </row>
+    <row r="489" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A489" s="13"/>
+    </row>
+    <row r="490" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A490" s="13"/>
+    </row>
+    <row r="491" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A491" s="13"/>
+    </row>
+    <row r="492" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A492" s="13"/>
+    </row>
+    <row r="493" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A493" s="13"/>
+    </row>
+    <row r="494" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A494" s="13"/>
+    </row>
+    <row r="495" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A495" s="13"/>
+    </row>
+    <row r="496" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A496" s="13"/>
+    </row>
+    <row r="497" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A497" s="13"/>
+    </row>
+    <row r="498" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A498" s="13"/>
+    </row>
+    <row r="499" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A499" s="13"/>
+    </row>
+    <row r="500" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A500" s="13"/>
+    </row>
+    <row r="501" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A501" s="13"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E3:E501" type="list">
+      <formula1>_listas!$F$1:$F$5</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="UTF-8" standalone="yes"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006"><sheetPr filterMode="false"><pageSetUpPr fitToPage="false"/></sheetPr><dimension ref="A1:I501"/><sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"></sheetFormatPr><cols><col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/><col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13"/><col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/><col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/><col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="46"/><col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16"/><col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/><col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="26"/><col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="34"/></cols><sheetData><row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"><c r="A1" s="6" t="s"><v>192</v></c><c r="B1" s="6" t="s"><v>84</v></c><c r="C1" s="6" t="s"><v>193</v></c><c r="D1" s="6" t="s"><v>194</v></c><c r="E1" s="6" t="s"><v>195</v></c><c r="F1" s="6" t="s"><v>168</v></c><c r="G1" s="6" t="s"><v>196</v></c><c r="H1" s="6" t="s"><v>197</v></c><c r="I1" s="6" t="s"><v>100</v></c></row><row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A2" s="22" t="s"><v>198</v></c><c r="B2" s="22" t="s"><v>199</v></c><c r="C2" s="22" t="s"><v>49</v></c><c r="D2" s="22" t="s"><v>200</v></c><c r="E2" s="22" t="s"><v>201</v></c><c r="F2" s="23" t="n"><v>15000</v></c><c r="G2" s="22" t="s"><v>50</v></c><c r="H2" s="22" t="s"><v>202</v></c><c r="I2" s="22" t="s"><v>106</v></c></row><row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A3" s="13"/><row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A4" s="13"/><row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A5" s="13"/><row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A6" s="13"/><row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A7" s="13"/><row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A8" s="13"/><row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A9" s="13"/><row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A10" s="13"/><row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A11" s="13"/><row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A12" s="13"/><row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A13" s="13"/><row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A14" s="13"/><row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A15" s="13"/><row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A16" s="13"/><row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A17" s="13"/><row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A18" s="13"/><row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A19" s="13"/><row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A20" s="13"/><row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A21" s="13"/><row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A22" s="13"/><row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A23" s="13"/><row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A24" s="13"/><row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A25" s="13"/><row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A26" s="13"/><row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A27" s="13"/><row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A28" s="13"/><row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A29" s="13"/><row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A30" s="13"/><row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A31" s="13"/><row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A32" s="13"/><row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A33" s="13"/><row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A34" s="13"/><row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A35" s="13"/><row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A36" s="13"/><row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A37" s="13"/><row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A38" s="13"/><row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A39" s="13"/><row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A40" s="13"/><row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A41" s="13"/><row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A42" s="13"/><row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A43" s="13"/><row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A44" s="13"/><row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A45" s="13"/><row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A46" s="13"/><row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A47" s="13"/><row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A48" s="13"/><row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A49" s="13"/><row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A50" s="13"/><row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A51" s="13"/><row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A52" s="13"/><row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A53" s="13"/><row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A54" s="13"/><row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A55" s="13"/><row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A56" s="13"/><row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A57" s="13"/><row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A58" s="13"/><row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A59" s="13"/><row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A60" s="13"/><row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A61" s="13"/><row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A62" s="13"/><row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A63" s="13"/><row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A64" s="13"/><row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A65" s="13"/><row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A66" s="13"/><row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A67" s="13"/><row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A68" s="13"/><row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A69" s="13"/><row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A70" s="13"/><row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A71" s="13"/><row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A72" s="13"/><row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A73" s="13"/><row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A74" s="13"/><row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A75" s="13"/><row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A76" s="13"/><row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A77" s="13"/><row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A78" s="13"/><row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A79" s="13"/><row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A80" s="13"/><row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A81" s="13"/><row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A82" s="13"/><row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A83" s="13"/><row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A84" s="13"/><row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A85" s="13"/><row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A86" s="13"/><row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A87" s="13"/><row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A88" s="13"/><row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A89" s="13"/><row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A90" s="13"/><row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A91" s="13"/><row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A92" s="13"/><row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A93" s="13"/><row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A94" s="13"/><row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A95" s="13"/><row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A96" s="13"/><row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A97" s="13"/><row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A98" s="13"/><row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A99" s="13"/><row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A100" s="13"/><row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A101" s="13"/><row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A102" s="13"/><row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A103" s="13"/><row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A104" s="13"/><row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A105" s="13"/><row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A106" s="13"/><row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A107" s="13"/><row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A108" s="13"/><row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A109" s="13"/><row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A110" s="13"/><row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A111" s="13"/><row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A112" s="13"/><row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A113" s="13"/><row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A114" s="13"/><row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A115" s="13"/><row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A116" s="13"/><row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A117" s="13"/><row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A118" s="13"/><row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A119" s="13"/><row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A120" s="13"/><row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A121" s="13"/><row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A122" s="13"/><row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A123" s="13"/><row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A124" s="13"/><row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A125" s="13"/><row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A126" s="13"/><row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A127" s="13"/><row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A128" s="13"/><row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A129" s="13"/><row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A130" s="13"/><row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A131" s="13"/><row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A132" s="13"/><row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A133" s="13"/><row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A134" s="13"/><row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A135" s="13"/><row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A136" s="13"/><row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A137" s="13"/><row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A138" s="13"/><row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A139" s="13"/><row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A140" s="13"/><row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A141" s="13"/><row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A142" s="13"/><row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A143" s="13"/><row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A144" s="13"/><row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A145" s="13"/><row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A146" s="13"/><row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A147" s="13"/><row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A148" s="13"/><row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A149" s="13"/><row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A150" s="13"/><row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A151" s="13"/><row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A152" s="13"/><row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A153" s="13"/><row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A154" s="13"/><row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A155" s="13"/><row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A156" s="13"/><row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A157" s="13"/><row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A158" s="13"/><row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A159" s="13"/><row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A160" s="13"/><row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A161" s="13"/><row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A162" s="13"/><row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A163" s="13"/><row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A164" s="13"/><row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A165" s="13"/><row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A166" s="13"/><row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A167" s="13"/><row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A168" s="13"/><row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A169" s="13"/><row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A170" s="13"/><row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A171" s="13"/><row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A172" s="13"/><row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A173" s="13"/><row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A174" s="13"/><row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A175" s="13"/><row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A176" s="13"/><row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A177" s="13"/><row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A178" s="13"/><row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A179" s="13"/><row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A180" s="13"/><row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A181" s="13"/><row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A182" s="13"/><row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A183" s="13"/><row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A184" s="13"/><row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A185" s="13"/><row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A186" s="13"/><row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A187" s="13"/><row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A188" s="13"/><row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A189" s="13"/><row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A190" s="13"/><row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A191" s="13"/><row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A192" s="13"/><row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A193" s="13"/><row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A194" s="13"/><row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A195" s="13"/><row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A196" s="13"/><row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A197" s="13"/><row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A198" s="13"/><row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A199" s="13"/><row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A200" s="13"/><row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A201" s="13"/><row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A202" s="13"/><row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A203" s="13"/><row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A204" s="13"/><row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A205" s="13"/><row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A206" s="13"/><row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A207" s="13"/><row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A208" s="13"/><row r="209" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A209" s="13"/><row r="210" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A210" s="13"/><row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A211" s="13"/><row r="212" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A212" s="13"/><row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A213" s="13"/><row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A214" s="13"/><row r="215" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A215" s="13"/><row r="216" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A216" s="13"/><row r="217" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A217" s="13"/><row r="218" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A218" s="13"/><row r="219" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A219" s="13"/><row r="220" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A220" s="13"/><row r="221" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A221" s="13"/><row r="222" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A222" s="13"/><row r="223" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A223" s="13"/><row r="224" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A224" s="13"/><row r="225" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A225" s="13"/><row r="226" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A226" s="13"/><row r="227" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A227" s="13"/><row r="228" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A228" s="13"/><row r="229" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A229" s="13"/><row r="230" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A230" s="13"/><row r="231" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A231" s="13"/><row r="232" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A232" s="13"/><row r="233" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A233" s="13"/><row r="234" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A234" s="13"/><row r="235" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A235" s="13"/><row r="236" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A236" s="13"/><row r="237" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A237" s="13"/><row r="238" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A238" s="13"/><row r="239" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A239" s="13"/><row r="240" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A240" s="13"/><row r="241" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A241" s="13"/><row r="242" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A242" s="13"/><row r="243" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A243" s="13"/><row r="244" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A244" s="13"/><row r="245" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A245" s="13"/><row r="246" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A246" s="13"/><row r="247" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A247" s="13"/><row r="248" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A248" s="13"/><row r="249" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A249" s="13"/><row r="250" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A250" s="13"/><row r="251" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A251" s="13"/><row r="252" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A252" s="13"/><row r="253" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A253" s="13"/><row r="254" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A254" s="13"/><row r="255" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A255" s="13"/><row r="256" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A256" s="13"/><row r="257" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A257" s="13"/><row r="258" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A258" s="13"/><row r="259" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A259" s="13"/><row r="260" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A260" s="13"/><row r="261" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A261" s="13"/><row r="262" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A262" s="13"/><row r="263" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A263" s="13"/><row r="264" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A264" s="13"/><row r="265" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A265" s="13"/><row r="266" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A266" s="13"/><row r="267" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A267" s="13"/><row r="268" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A268" s="13"/><row r="269" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A269" s="13"/><row r="270" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A270" s="13"/><row r="271" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A271" s="13"/><row r="272" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A272" s="13"/><row r="273" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A273" s="13"/><row r="274" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A274" s="13"/><row r="275" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A275" s="13"/><row r="276" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A276" s="13"/><row r="277" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A277" s="13"/><row r="278" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A278" s="13"/><row r="279" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A279" s="13"/><row r="280" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A280" s="13"/><row r="281" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A281" s="13"/><row r="282" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A282" s="13"/><row r="283" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A283" s="13"/><row r="284" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A284" s="13"/><row r="285" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A285" s="13"/><row r="286" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A286" s="13"/><row r="287" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A287" s="13"/><row r="288" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A288" s="13"/><row r="289" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A289" s="13"/><row r="290" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A290" s="13"/><row r="291" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A291" s="13"/><row r="292" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A292" s="13"/><row r="293" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A293" s="13"/><row r="294" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A294" s="13"/><row r="295" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A295" s="13"/><row r="296" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A296" s="13"/><row r="297" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A297" s="13"/><row r="298" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A298" s="13"/><row r="299" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A299" s="13"/><row r="300" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A300" s="13"/><row r="301" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A301" s="13"/><row r="302" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A302" s="13"/><row r="303" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A303" s="13"/><row r="304" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A304" s="13"/><row r="305" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A305" s="13"/><row r="306" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A306" s="13"/><row r="307" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A307" s="13"/><row r="308" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A308" s="13"/><row r="309" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A309" s="13"/><row r="310" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A310" s="13"/><row r="311" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A311" s="13"/><row r="312" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A312" s="13"/><row r="313" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A313" s="13"/><row r="314" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A314" s="13"/><row r="315" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A315" s="13"/><row r="316" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A316" s="13"/><row r="317" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A317" s="13"/><row r="318" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A318" s="13"/><row r="319" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A319" s="13"/><row r="320" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A320" s="13"/><row r="321" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A321" s="13"/><row r="322" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A322" s="13"/><row r="323" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A323" s="13"/><row r="324" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A324" s="13"/><row r="325" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A325" s="13"/><row r="326" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A326" s="13"/><row r="327" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A327" s="13"/><row r="328" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A328" s="13"/><row r="329" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A329" s="13"/><row r="330" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A330" s="13"/><row r="331" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A331" s="13"/><row r="332" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A332" s="13"/><row r="333" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A333" s="13"/><row r="334" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A334" s="13"/><row r="335" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A335" s="13"/><row r="336" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A336" s="13"/><row r="337" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A337" s="13"/><row r="338" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A338" s="13"/><row r="339" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A339" s="13"/><row r="340" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A340" s="13"/><row r="341" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A341" s="13"/><row r="342" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A342" s="13"/><row r="343" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A343" s="13"/><row r="344" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A344" s="13"/><row r="345" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A345" s="13"/><row r="346" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A346" s="13"/><row r="347" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A347" s="13"/><row r="348" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A348" s="13"/><row r="349" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A349" s="13"/><row r="350" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A350" s="13"/><row r="351" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A351" s="13"/><row r="352" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A352" s="13"/><row r="353" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A353" s="13"/><row r="354" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A354" s="13"/><row r="355" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A355" s="13"/><row r="356" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A356" s="13"/><row r="357" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A357" s="13"/><row r="358" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A358" s="13"/><row r="359" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A359" s="13"/><row r="360" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A360" s="13"/><row r="361" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A361" s="13"/><row r="362" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A362" s="13"/><row r="363" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A363" s="13"/><row r="364" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A364" s="13"/><row r="365" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A365" s="13"/><row r="366" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A366" s="13"/><row r="367" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A367" s="13"/><row r="368" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A368" s="13"/><row r="369" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A369" s="13"/><row r="370" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A370" s="13"/><row r="371" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A371" s="13"/><row r="372" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A372" s="13"/><row r="373" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A373" s="13"/><row r="374" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A374" s="13"/><row r="375" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A375" s="13"/><row r="376" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A376" s="13"/><row r="377" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A377" s="13"/><row r="378" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A378" s="13"/><row r="379" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A379" s="13"/><row r="380" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A380" s="13"/><row r="381" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A381" s="13"/><row r="382" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A382" s="13"/><row r="383" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A383" s="13"/><row r="384" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A384" s="13"/><row r="385" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A385" s="13"/><row r="386" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A386" s="13"/><row r="387" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A387" s="13"/><row r="388" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A388" s="13"/><row r="389" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A389" s="13"/><row r="390" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A390" s="13"/><row r="391" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A391" s="13"/><row r="392" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A392" s="13"/><row r="393" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A393" s="13"/><row r="394" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A394" s="13"/><row r="395" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A395" s="13"/><row r="396" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A396" s="13"/><row r="397" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A397" s="13"/><row r="398" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A398" s="13"/><row r="399" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A399" s="13"/><row r="400" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A400" s="13"/><row r="401" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A401" s="13"/><row r="402" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A402" s="13"/><row r="403" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A403" s="13"/><row r="404" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A404" s="13"/><row r="405" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A405" s="13"/><row r="406" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A406" s="13"/><row r="407" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A407" s="13"/><row r="408" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A408" s="13"/><row r="409" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A409" s="13"/><row r="410" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A410" s="13"/><row r="411" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A411" s="13"/><row r="412" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A412" s="13"/><row r="413" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A413" s="13"/><row r="414" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A414" s="13"/><row r="415" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A415" s="13"/><row r="416" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A416" s="13"/><row r="417" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A417" s="13"/><row r="418" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A418" s="13"/><row r="419" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A419" s="13"/><row r="420" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A420" s="13"/><row r="421" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A421" s="13"/><row r="422" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A422" s="13"/><row r="423" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A423" s="13"/><row r="424" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A424" s="13"/><row r="425" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A425" s="13"/><row r="426" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A426" s="13"/><row r="427" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A427" s="13"/><row r="428" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A428" s="13"/><row r="429" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A429" s="13"/><row r="430" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A430" s="13"/><row r="431" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A431" s="13"/><row r="432" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A432" s="13"/><row r="433" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A433" s="13"/><row r="434" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A434" s="13"/><row r="435" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A435" s="13"/><row r="436" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A436" s="13"/><row r="437" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A437" s="13"/><row r="438" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A438" s="13"/><row r="439" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A439" s="13"/><row r="440" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A440" s="13"/><row r="441" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A441" s="13"/><row r="442" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A442" s="13"/><row r="443" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A443" s="13"/><row r="444" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A444" s="13"/><row r="445" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A445" s="13"/><row r="446" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A446" s="13"/><row r="447" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A447" s="13"/><row r="448" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A448" s="13"/><row r="449" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A449" s="13"/><row r="450" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A450" s="13"/><row r="451" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A451" s="13"/><row r="452" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A452" s="13"/><row r="453" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A453" s="13"/><row r="454" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A454" s="13"/><row r="455" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A455" s="13"/><row r="456" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A456" s="13"/><row r="457" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A457" s="13"/><row r="458" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A458" s="13"/><row r="459" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A459" s="13"/><row r="460" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A460" s="13"/><row r="461" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A461" s="13"/><row r="462" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A462" s="13"/><row r="463" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A463" s="13"/><row r="464" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A464" s="13"/><row r="465" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A465" s="13"/><row r="466" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A466" s="13"/><row r="467" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A467" s="13"/><row r="468" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A468" s="13"/><row r="469" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A469" s="13"/><row r="470" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A470" s="13"/><row r="471" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A471" s="13"/><row r="472" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A472" s="13"/><row r="473" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A473" s="13"/><row r="474" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A474" s="13"/><row r="475" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A475" s="13"/><row r="476" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A476" s="13"/><row r="477" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A477" s="13"/><row r="478" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A478" s="13"/><row r="479" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A479" s="13"/><row r="480" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A480" s="13"/><row r="481" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A481" s="13"/><row r="482" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A482" s="13"/><row r="483" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A483" s="13"/><row r="484" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A484" s="13"/><row r="485" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A485" s="13"/><row r="486" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A486" s="13"/><row r="487" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A487" s="13"/><row r="488" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A488" s="13"/><row r="489" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A489" s="13"/><row r="490" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A490" s="13"/><row r="491" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A491" s="13"/><row r="492" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A492" s="13"/><row r="493" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A493" s="13"/><row r="494" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A494" s="13"/><row r="495" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A495" s="13"/><row r="496" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A496" s="13"/><row r="497" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A497" s="13"/><row r="498" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A498" s="13"/><row r="499" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A499" s="13"/><row r="500" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A500" s="13"/><row r="501" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"><c r="A501" s="13"/></sheetData><dataValidations count="2"><dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C3:C501" type="list"><formula1>_listas!$E$1:$E$11</formula1><formula2>0</formula2></dataValidation><dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G3:G501" type="list"><formula1>_listas!$F$1:$F$2</formula1><formula2>0</formula2></dataValidation></dataValidations><printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/><pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/><pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/><headerFooter differentFirst="false" differentOddEven="false"><oddHeader></oddHeader><oddFooter></oddFooter></headerFooter></worksheet>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:I501"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="34"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="22" t="s">
+        <v>198</v>
+      </c>
+      <c r="B2" s="22" t="s">
+        <v>199</v>
+      </c>
+      <c r="C2" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2" s="22" t="s">
+        <v>200</v>
+      </c>
+      <c r="E2" s="22" t="s">
+        <v>201</v>
+      </c>
+      <c r="F2" s="23" t="n">
+        <v>15000</v>
+      </c>
+      <c r="G2" s="22" t="s">
+        <v>50</v>
+      </c>
+      <c r="H2" s="22" t="s">
+        <v>202</v>
+      </c>
+      <c r="I2" s="22" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="13"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="13"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="13"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="13"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="13"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="13"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="13"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="13"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="13"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="13"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="13"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="13"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="13"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="13"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="13"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="13"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="13"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="13"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="13"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="13"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="13"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="13"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="13"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="13"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="13"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="13"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="13"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="13"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="13"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="13"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="13"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="13"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="13"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="13"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="13"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="13"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="13"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="13"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="13"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="13"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="13"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="13"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="13"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="13"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="13"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="13"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="13"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="13"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="13"/>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="13"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="13"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="13"/>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="13"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="13"/>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="13"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="13"/>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="13"/>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="13"/>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="13"/>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="13"/>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="13"/>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="13"/>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="13"/>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="13"/>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="13"/>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="13"/>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="13"/>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="13"/>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="13"/>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="13"/>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="13"/>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="13"/>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="13"/>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="13"/>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="13"/>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="13"/>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="13"/>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="13"/>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="13"/>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="13"/>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="13"/>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="13"/>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="13"/>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="13"/>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="13"/>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="13"/>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="13"/>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="13"/>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="13"/>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="13"/>
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="13"/>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="13"/>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="13"/>
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="13"/>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="13"/>
+    </row>
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="13"/>
+    </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="13"/>
+    </row>
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="13"/>
+    </row>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="13"/>
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="13"/>
+    </row>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="13"/>
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="13"/>
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="13"/>
+    </row>
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="13"/>
+    </row>
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="13"/>
+    </row>
+    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="13"/>
+    </row>
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="13"/>
+    </row>
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="13"/>
+    </row>
+    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="13"/>
+    </row>
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="13"/>
+    </row>
+    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="13"/>
+    </row>
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="13"/>
+    </row>
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="13"/>
+    </row>
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="13"/>
+    </row>
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="13"/>
+    </row>
+    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="13"/>
+    </row>
+    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="13"/>
+    </row>
+    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="13"/>
+    </row>
+    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A121" s="13"/>
+    </row>
+    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A122" s="13"/>
+    </row>
+    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A123" s="13"/>
+    </row>
+    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A124" s="13"/>
+    </row>
+    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A125" s="13"/>
+    </row>
+    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A126" s="13"/>
+    </row>
+    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A127" s="13"/>
+    </row>
+    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A128" s="13"/>
+    </row>
+    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A129" s="13"/>
+    </row>
+    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A130" s="13"/>
+    </row>
+    <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A131" s="13"/>
+    </row>
+    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A132" s="13"/>
+    </row>
+    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A133" s="13"/>
+    </row>
+    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A134" s="13"/>
+    </row>
+    <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A135" s="13"/>
+    </row>
+    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A136" s="13"/>
+    </row>
+    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A137" s="13"/>
+    </row>
+    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A138" s="13"/>
+    </row>
+    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A139" s="13"/>
+    </row>
+    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A140" s="13"/>
+    </row>
+    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A141" s="13"/>
+    </row>
+    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A142" s="13"/>
+    </row>
+    <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A143" s="13"/>
+    </row>
+    <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A144" s="13"/>
+    </row>
+    <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A145" s="13"/>
+    </row>
+    <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A146" s="13"/>
+    </row>
+    <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A147" s="13"/>
+    </row>
+    <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A148" s="13"/>
+    </row>
+    <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A149" s="13"/>
+    </row>
+    <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A150" s="13"/>
+    </row>
+    <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A151" s="13"/>
+    </row>
+    <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A152" s="13"/>
+    </row>
+    <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A153" s="13"/>
+    </row>
+    <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A154" s="13"/>
+    </row>
+    <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A155" s="13"/>
+    </row>
+    <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A156" s="13"/>
+    </row>
+    <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A157" s="13"/>
+    </row>
+    <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A158" s="13"/>
+    </row>
+    <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A159" s="13"/>
+    </row>
+    <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A160" s="13"/>
+    </row>
+    <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A161" s="13"/>
+    </row>
+    <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A162" s="13"/>
+    </row>
+    <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A163" s="13"/>
+    </row>
+    <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A164" s="13"/>
+    </row>
+    <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A165" s="13"/>
+    </row>
+    <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A166" s="13"/>
+    </row>
+    <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A167" s="13"/>
+    </row>
+    <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A168" s="13"/>
+    </row>
+    <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A169" s="13"/>
+    </row>
+    <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A170" s="13"/>
+    </row>
+    <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A171" s="13"/>
+    </row>
+    <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A172" s="13"/>
+    </row>
+    <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A173" s="13"/>
+    </row>
+    <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A174" s="13"/>
+    </row>
+    <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A175" s="13"/>
+    </row>
+    <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A176" s="13"/>
+    </row>
+    <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A177" s="13"/>
+    </row>
+    <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A178" s="13"/>
+    </row>
+    <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A179" s="13"/>
+    </row>
+    <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A180" s="13"/>
+    </row>
+    <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A181" s="13"/>
+    </row>
+    <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A182" s="13"/>
+    </row>
+    <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A183" s="13"/>
+    </row>
+    <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A184" s="13"/>
+    </row>
+    <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A185" s="13"/>
+    </row>
+    <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A186" s="13"/>
+    </row>
+    <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A187" s="13"/>
+    </row>
+    <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A188" s="13"/>
+    </row>
+    <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A189" s="13"/>
+    </row>
+    <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A190" s="13"/>
+    </row>
+    <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A191" s="13"/>
+    </row>
+    <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A192" s="13"/>
+    </row>
+    <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A193" s="13"/>
+    </row>
+    <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A194" s="13"/>
+    </row>
+    <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A195" s="13"/>
+    </row>
+    <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A196" s="13"/>
+    </row>
+    <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A197" s="13"/>
+    </row>
+    <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A198" s="13"/>
+    </row>
+    <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A199" s="13"/>
+    </row>
+    <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A200" s="13"/>
+    </row>
+    <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A201" s="13"/>
+    </row>
+    <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A202" s="13"/>
+    </row>
+    <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A203" s="13"/>
+    </row>
+    <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A204" s="13"/>
+    </row>
+    <row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A205" s="13"/>
+    </row>
+    <row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A206" s="13"/>
+    </row>
+    <row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A207" s="13"/>
+    </row>
+    <row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A208" s="13"/>
+    </row>
+    <row r="209" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A209" s="13"/>
+    </row>
+    <row r="210" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A210" s="13"/>
+    </row>
+    <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A211" s="13"/>
+    </row>
+    <row r="212" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A212" s="13"/>
+    </row>
+    <row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A213" s="13"/>
+    </row>
+    <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A214" s="13"/>
+    </row>
+    <row r="215" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A215" s="13"/>
+    </row>
+    <row r="216" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A216" s="13"/>
+    </row>
+    <row r="217" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A217" s="13"/>
+    </row>
+    <row r="218" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A218" s="13"/>
+    </row>
+    <row r="219" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A219" s="13"/>
+    </row>
+    <row r="220" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A220" s="13"/>
+    </row>
+    <row r="221" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A221" s="13"/>
+    </row>
+    <row r="222" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A222" s="13"/>
+    </row>
+    <row r="223" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A223" s="13"/>
+    </row>
+    <row r="224" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A224" s="13"/>
+    </row>
+    <row r="225" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A225" s="13"/>
+    </row>
+    <row r="226" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A226" s="13"/>
+    </row>
+    <row r="227" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A227" s="13"/>
+    </row>
+    <row r="228" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A228" s="13"/>
+    </row>
+    <row r="229" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A229" s="13"/>
+    </row>
+    <row r="230" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A230" s="13"/>
+    </row>
+    <row r="231" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A231" s="13"/>
+    </row>
+    <row r="232" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A232" s="13"/>
+    </row>
+    <row r="233" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A233" s="13"/>
+    </row>
+    <row r="234" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A234" s="13"/>
+    </row>
+    <row r="235" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A235" s="13"/>
+    </row>
+    <row r="236" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A236" s="13"/>
+    </row>
+    <row r="237" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A237" s="13"/>
+    </row>
+    <row r="238" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A238" s="13"/>
+    </row>
+    <row r="239" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A239" s="13"/>
+    </row>
+    <row r="240" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A240" s="13"/>
+    </row>
+    <row r="241" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A241" s="13"/>
+    </row>
+    <row r="242" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A242" s="13"/>
+    </row>
+    <row r="243" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A243" s="13"/>
+    </row>
+    <row r="244" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A244" s="13"/>
+    </row>
+    <row r="245" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A245" s="13"/>
+    </row>
+    <row r="246" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A246" s="13"/>
+    </row>
+    <row r="247" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A247" s="13"/>
+    </row>
+    <row r="248" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A248" s="13"/>
+    </row>
+    <row r="249" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A249" s="13"/>
+    </row>
+    <row r="250" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A250" s="13"/>
+    </row>
+    <row r="251" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A251" s="13"/>
+    </row>
+    <row r="252" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A252" s="13"/>
+    </row>
+    <row r="253" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A253" s="13"/>
+    </row>
+    <row r="254" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A254" s="13"/>
+    </row>
+    <row r="255" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A255" s="13"/>
+    </row>
+    <row r="256" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A256" s="13"/>
+    </row>
+    <row r="257" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A257" s="13"/>
+    </row>
+    <row r="258" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A258" s="13"/>
+    </row>
+    <row r="259" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A259" s="13"/>
+    </row>
+    <row r="260" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A260" s="13"/>
+    </row>
+    <row r="261" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A261" s="13"/>
+    </row>
+    <row r="262" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A262" s="13"/>
+    </row>
+    <row r="263" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A263" s="13"/>
+    </row>
+    <row r="264" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A264" s="13"/>
+    </row>
+    <row r="265" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A265" s="13"/>
+    </row>
+    <row r="266" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A266" s="13"/>
+    </row>
+    <row r="267" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A267" s="13"/>
+    </row>
+    <row r="268" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A268" s="13"/>
+    </row>
+    <row r="269" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A269" s="13"/>
+    </row>
+    <row r="270" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A270" s="13"/>
+    </row>
+    <row r="271" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A271" s="13"/>
+    </row>
+    <row r="272" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A272" s="13"/>
+    </row>
+    <row r="273" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A273" s="13"/>
+    </row>
+    <row r="274" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A274" s="13"/>
+    </row>
+    <row r="275" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A275" s="13"/>
+    </row>
+    <row r="276" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A276" s="13"/>
+    </row>
+    <row r="277" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A277" s="13"/>
+    </row>
+    <row r="278" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A278" s="13"/>
+    </row>
+    <row r="279" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A279" s="13"/>
+    </row>
+    <row r="280" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A280" s="13"/>
+    </row>
+    <row r="281" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A281" s="13"/>
+    </row>
+    <row r="282" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A282" s="13"/>
+    </row>
+    <row r="283" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A283" s="13"/>
+    </row>
+    <row r="284" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A284" s="13"/>
+    </row>
+    <row r="285" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A285" s="13"/>
+    </row>
+    <row r="286" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A286" s="13"/>
+    </row>
+    <row r="287" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A287" s="13"/>
+    </row>
+    <row r="288" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A288" s="13"/>
+    </row>
+    <row r="289" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A289" s="13"/>
+    </row>
+    <row r="290" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A290" s="13"/>
+    </row>
+    <row r="291" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A291" s="13"/>
+    </row>
+    <row r="292" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A292" s="13"/>
+    </row>
+    <row r="293" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A293" s="13"/>
+    </row>
+    <row r="294" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A294" s="13"/>
+    </row>
+    <row r="295" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A295" s="13"/>
+    </row>
+    <row r="296" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A296" s="13"/>
+    </row>
+    <row r="297" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A297" s="13"/>
+    </row>
+    <row r="298" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A298" s="13"/>
+    </row>
+    <row r="299" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A299" s="13"/>
+    </row>
+    <row r="300" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A300" s="13"/>
+    </row>
+    <row r="301" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A301" s="13"/>
+    </row>
+    <row r="302" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A302" s="13"/>
+    </row>
+    <row r="303" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A303" s="13"/>
+    </row>
+    <row r="304" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A304" s="13"/>
+    </row>
+    <row r="305" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A305" s="13"/>
+    </row>
+    <row r="306" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A306" s="13"/>
+    </row>
+    <row r="307" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A307" s="13"/>
+    </row>
+    <row r="308" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A308" s="13"/>
+    </row>
+    <row r="309" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A309" s="13"/>
+    </row>
+    <row r="310" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A310" s="13"/>
+    </row>
+    <row r="311" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A311" s="13"/>
+    </row>
+    <row r="312" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A312" s="13"/>
+    </row>
+    <row r="313" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A313" s="13"/>
+    </row>
+    <row r="314" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A314" s="13"/>
+    </row>
+    <row r="315" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A315" s="13"/>
+    </row>
+    <row r="316" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A316" s="13"/>
+    </row>
+    <row r="317" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A317" s="13"/>
+    </row>
+    <row r="318" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A318" s="13"/>
+    </row>
+    <row r="319" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A319" s="13"/>
+    </row>
+    <row r="320" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A320" s="13"/>
+    </row>
+    <row r="321" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A321" s="13"/>
+    </row>
+    <row r="322" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A322" s="13"/>
+    </row>
+    <row r="323" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A323" s="13"/>
+    </row>
+    <row r="324" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A324" s="13"/>
+    </row>
+    <row r="325" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A325" s="13"/>
+    </row>
+    <row r="326" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A326" s="13"/>
+    </row>
+    <row r="327" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A327" s="13"/>
+    </row>
+    <row r="328" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A328" s="13"/>
+    </row>
+    <row r="329" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A329" s="13"/>
+    </row>
+    <row r="330" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A330" s="13"/>
+    </row>
+    <row r="331" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A331" s="13"/>
+    </row>
+    <row r="332" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A332" s="13"/>
+    </row>
+    <row r="333" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A333" s="13"/>
+    </row>
+    <row r="334" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A334" s="13"/>
+    </row>
+    <row r="335" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A335" s="13"/>
+    </row>
+    <row r="336" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A336" s="13"/>
+    </row>
+    <row r="337" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A337" s="13"/>
+    </row>
+    <row r="338" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A338" s="13"/>
+    </row>
+    <row r="339" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A339" s="13"/>
+    </row>
+    <row r="340" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A340" s="13"/>
+    </row>
+    <row r="341" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A341" s="13"/>
+    </row>
+    <row r="342" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A342" s="13"/>
+    </row>
+    <row r="343" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A343" s="13"/>
+    </row>
+    <row r="344" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A344" s="13"/>
+    </row>
+    <row r="345" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A345" s="13"/>
+    </row>
+    <row r="346" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A346" s="13"/>
+    </row>
+    <row r="347" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A347" s="13"/>
+    </row>
+    <row r="348" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A348" s="13"/>
+    </row>
+    <row r="349" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A349" s="13"/>
+    </row>
+    <row r="350" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A350" s="13"/>
+    </row>
+    <row r="351" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A351" s="13"/>
+    </row>
+    <row r="352" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A352" s="13"/>
+    </row>
+    <row r="353" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A353" s="13"/>
+    </row>
+    <row r="354" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A354" s="13"/>
+    </row>
+    <row r="355" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A355" s="13"/>
+    </row>
+    <row r="356" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A356" s="13"/>
+    </row>
+    <row r="357" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A357" s="13"/>
+    </row>
+    <row r="358" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A358" s="13"/>
+    </row>
+    <row r="359" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A359" s="13"/>
+    </row>
+    <row r="360" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A360" s="13"/>
+    </row>
+    <row r="361" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A361" s="13"/>
+    </row>
+    <row r="362" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A362" s="13"/>
+    </row>
+    <row r="363" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A363" s="13"/>
+    </row>
+    <row r="364" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A364" s="13"/>
+    </row>
+    <row r="365" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A365" s="13"/>
+    </row>
+    <row r="366" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A366" s="13"/>
+    </row>
+    <row r="367" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A367" s="13"/>
+    </row>
+    <row r="368" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A368" s="13"/>
+    </row>
+    <row r="369" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A369" s="13"/>
+    </row>
+    <row r="370" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A370" s="13"/>
+    </row>
+    <row r="371" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A371" s="13"/>
+    </row>
+    <row r="372" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A372" s="13"/>
+    </row>
+    <row r="373" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A373" s="13"/>
+    </row>
+    <row r="374" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A374" s="13"/>
+    </row>
+    <row r="375" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A375" s="13"/>
+    </row>
+    <row r="376" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A376" s="13"/>
+    </row>
+    <row r="377" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A377" s="13"/>
+    </row>
+    <row r="378" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A378" s="13"/>
+    </row>
+    <row r="379" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A379" s="13"/>
+    </row>
+    <row r="380" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A380" s="13"/>
+    </row>
+    <row r="381" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A381" s="13"/>
+    </row>
+    <row r="382" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A382" s="13"/>
+    </row>
+    <row r="383" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A383" s="13"/>
+    </row>
+    <row r="384" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A384" s="13"/>
+    </row>
+    <row r="385" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A385" s="13"/>
+    </row>
+    <row r="386" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A386" s="13"/>
+    </row>
+    <row r="387" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A387" s="13"/>
+    </row>
+    <row r="388" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A388" s="13"/>
+    </row>
+    <row r="389" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A389" s="13"/>
+    </row>
+    <row r="390" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A390" s="13"/>
+    </row>
+    <row r="391" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A391" s="13"/>
+    </row>
+    <row r="392" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A392" s="13"/>
+    </row>
+    <row r="393" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A393" s="13"/>
+    </row>
+    <row r="394" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A394" s="13"/>
+    </row>
+    <row r="395" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A395" s="13"/>
+    </row>
+    <row r="396" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A396" s="13"/>
+    </row>
+    <row r="397" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A397" s="13"/>
+    </row>
+    <row r="398" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A398" s="13"/>
+    </row>
+    <row r="399" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A399" s="13"/>
+    </row>
+    <row r="400" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A400" s="13"/>
+    </row>
+    <row r="401" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A401" s="13"/>
+    </row>
+    <row r="402" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A402" s="13"/>
+    </row>
+    <row r="403" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A403" s="13"/>
+    </row>
+    <row r="404" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A404" s="13"/>
+    </row>
+    <row r="405" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A405" s="13"/>
+    </row>
+    <row r="406" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A406" s="13"/>
+    </row>
+    <row r="407" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A407" s="13"/>
+    </row>
+    <row r="408" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A408" s="13"/>
+    </row>
+    <row r="409" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A409" s="13"/>
+    </row>
+    <row r="410" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A410" s="13"/>
+    </row>
+    <row r="411" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A411" s="13"/>
+    </row>
+    <row r="412" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A412" s="13"/>
+    </row>
+    <row r="413" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A413" s="13"/>
+    </row>
+    <row r="414" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A414" s="13"/>
+    </row>
+    <row r="415" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A415" s="13"/>
+    </row>
+    <row r="416" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A416" s="13"/>
+    </row>
+    <row r="417" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A417" s="13"/>
+    </row>
+    <row r="418" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A418" s="13"/>
+    </row>
+    <row r="419" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A419" s="13"/>
+    </row>
+    <row r="420" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A420" s="13"/>
+    </row>
+    <row r="421" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A421" s="13"/>
+    </row>
+    <row r="422" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A422" s="13"/>
+    </row>
+    <row r="423" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A423" s="13"/>
+    </row>
+    <row r="424" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A424" s="13"/>
+    </row>
+    <row r="425" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A425" s="13"/>
+    </row>
+    <row r="426" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A426" s="13"/>
+    </row>
+    <row r="427" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A427" s="13"/>
+    </row>
+    <row r="428" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A428" s="13"/>
+    </row>
+    <row r="429" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A429" s="13"/>
+    </row>
+    <row r="430" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A430" s="13"/>
+    </row>
+    <row r="431" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A431" s="13"/>
+    </row>
+    <row r="432" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A432" s="13"/>
+    </row>
+    <row r="433" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A433" s="13"/>
+    </row>
+    <row r="434" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A434" s="13"/>
+    </row>
+    <row r="435" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A435" s="13"/>
+    </row>
+    <row r="436" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A436" s="13"/>
+    </row>
+    <row r="437" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A437" s="13"/>
+    </row>
+    <row r="438" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A438" s="13"/>
+    </row>
+    <row r="439" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A439" s="13"/>
+    </row>
+    <row r="440" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A440" s="13"/>
+    </row>
+    <row r="441" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A441" s="13"/>
+    </row>
+    <row r="442" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A442" s="13"/>
+    </row>
+    <row r="443" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A443" s="13"/>
+    </row>
+    <row r="444" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A444" s="13"/>
+    </row>
+    <row r="445" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A445" s="13"/>
+    </row>
+    <row r="446" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A446" s="13"/>
+    </row>
+    <row r="447" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A447" s="13"/>
+    </row>
+    <row r="448" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A448" s="13"/>
+    </row>
+    <row r="449" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A449" s="13"/>
+    </row>
+    <row r="450" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A450" s="13"/>
+    </row>
+    <row r="451" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A451" s="13"/>
+    </row>
+    <row r="452" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A452" s="13"/>
+    </row>
+    <row r="453" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A453" s="13"/>
+    </row>
+    <row r="454" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A454" s="13"/>
+    </row>
+    <row r="455" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A455" s="13"/>
+    </row>
+    <row r="456" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A456" s="13"/>
+    </row>
+    <row r="457" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A457" s="13"/>
+    </row>
+    <row r="458" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A458" s="13"/>
+    </row>
+    <row r="459" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A459" s="13"/>
+    </row>
+    <row r="460" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A460" s="13"/>
+    </row>
+    <row r="461" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A461" s="13"/>
+    </row>
+    <row r="462" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A462" s="13"/>
+    </row>
+    <row r="463" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A463" s="13"/>
+    </row>
+    <row r="464" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A464" s="13"/>
+    </row>
+    <row r="465" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A465" s="13"/>
+    </row>
+    <row r="466" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A466" s="13"/>
+    </row>
+    <row r="467" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A467" s="13"/>
+    </row>
+    <row r="468" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A468" s="13"/>
+    </row>
+    <row r="469" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A469" s="13"/>
+    </row>
+    <row r="470" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A470" s="13"/>
+    </row>
+    <row r="471" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A471" s="13"/>
+    </row>
+    <row r="472" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A472" s="13"/>
+    </row>
+    <row r="473" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A473" s="13"/>
+    </row>
+    <row r="474" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A474" s="13"/>
+    </row>
+    <row r="475" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A475" s="13"/>
+    </row>
+    <row r="476" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A476" s="13"/>
+    </row>
+    <row r="477" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A477" s="13"/>
+    </row>
+    <row r="478" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A478" s="13"/>
+    </row>
+    <row r="479" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A479" s="13"/>
+    </row>
+    <row r="480" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A480" s="13"/>
+    </row>
+    <row r="481" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A481" s="13"/>
+    </row>
+    <row r="482" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A482" s="13"/>
+    </row>
+    <row r="483" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A483" s="13"/>
+    </row>
+    <row r="484" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A484" s="13"/>
+    </row>
+    <row r="485" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A485" s="13"/>
+    </row>
+    <row r="486" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A486" s="13"/>
+    </row>
+    <row r="487" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A487" s="13"/>
+    </row>
+    <row r="488" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A488" s="13"/>
+    </row>
+    <row r="489" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A489" s="13"/>
+    </row>
+    <row r="490" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A490" s="13"/>
+    </row>
+    <row r="491" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A491" s="13"/>
+    </row>
+    <row r="492" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A492" s="13"/>
+    </row>
+    <row r="493" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A493" s="13"/>
+    </row>
+    <row r="494" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A494" s="13"/>
+    </row>
+    <row r="495" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A495" s="13"/>
+    </row>
+    <row r="496" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A496" s="13"/>
+    </row>
+    <row r="497" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A497" s="13"/>
+    </row>
+    <row r="498" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A498" s="13"/>
+    </row>
+    <row r="499" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A499" s="13"/>
+    </row>
+    <row r="500" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A500" s="13"/>
+    </row>
+    <row r="501" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A501" s="13"/>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C3:C501" type="list">
+      <formula1>_listas!$D$1:$D$11</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G3:G501" type="list">
+      <formula1>_listas!$E$1:$E$2</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
fix: valida la hoja parametros como capa
</commit_message>
<xml_diff>
--- a/docs/Plantilla_Captura_Reporteria_v1.xlsx
+++ b/docs/Plantilla_Captura_Reporteria_v1.xlsx
@@ -1405,12 +1405,14 @@
         <v>24</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C19" s="3" t="s">
-        <v>26</v>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Configuracion general: moneda, IVA, tasa de provision. Se llena una sola vez. Porcentajes: 30%, 30 y 0.30 valen lo mismo; un numero mayor que 1 se lee como por ciento, y 1 solo es 100% (para uno por ciento escriba 1%). Fechas en dd/mm/aaaa.</t>
+        </is>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5919,15 +5921,17 @@
         <v>225</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="20" t="s">
         <v>226</v>
       </c>
       <c r="B4" s="16" t="n">
         <v>0.16</v>
       </c>
-      <c r="C4" s="24" t="s">
-        <v>227</v>
+      <c r="C4" s="24" t="inlineStr">
+        <is>
+          <t>Tasa aplicable. Porcentaje: 16%, 16 o 0.16 valen lo mismo; un numero mayor que 1 se lee como por ciento.</t>
+        </is>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5970,26 +5974,30 @@
         <v>237</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="20" t="s">
         <v>238</v>
       </c>
       <c r="B9" s="16" t="n">
         <v>0.25</v>
       </c>
-      <c r="C9" s="24" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C9" s="24" t="inlineStr">
+        <is>
+          <t>% de la cartera de 91-180 dias que se estima incobrable. Porcentaje: 25%, 25 o 0.25; un numero mayor que 1 se lee como por ciento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
         <v>240</v>
       </c>
       <c r="B10" s="16" t="n">
         <v>0.5</v>
       </c>
-      <c r="C10" s="24" t="s">
-        <v>241</v>
+      <c r="C10" s="24" t="inlineStr">
+        <is>
+          <t>% de la cartera de mas de 180 dias que se estima incobrable. Porcentaje: 50%, 50 o 0.50; un numero mayor que 1 se lee como por ciento.</t>
+        </is>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
fix: la hoja INSTRUCCIONES deja de prometer fórmulas que la plantilla no trae
</commit_message>
<xml_diff>
--- a/docs/Plantilla_Captura_Reporteria_v1.xlsx
+++ b/docs/Plantilla_Captura_Reporteria_v1.xlsx
@@ -1321,12 +1321,14 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>7</v>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Solo escriba en las celdas de LETRA AZUL. Las columnas de letra negra (utilidad, margen, cobrado y saldo) no se capturan: traen formula solo en la fila de ejemplo, y la aplicacion las calcula al cargar el archivo.</t>
+        </is>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1479,8 +1481,10 @@
       <c r="B29" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C29" s="3" t="s">
-        <v>40</v>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Columna calculada por la aplicacion al cargar el archivo. No escriba en ella.</t>
+        </is>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>